<commit_message>
Update PropExcel_Test_Cases.xlsx with new test scenarios and data adjustment
</commit_message>
<xml_diff>
--- a/PropExcel_Test_Cases.xlsx
+++ b/PropExcel_Test_Cases.xlsx
@@ -10,6 +10,9 @@
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="TC-01_Flow1" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="TC-02_Flow2" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="TC-03_CreateOrganization" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="TC-04_Flow1_NewOrg" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="TC-05_Flow2_NewOrg" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,6 +40,11 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E78"/>
+      <sz val="14"/>
     </font>
   </fonts>
   <fills count="4">
@@ -57,7 +65,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -79,11 +87,25 @@
         <color rgb="00B7B7B7"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B0B0B0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -97,6 +119,17 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -463,15 +496,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
     <col width="110" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>PropExcel Automated Test Cases</t>
         </is>
@@ -509,7 +542,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>test240</t>
+          <t>Legacy: test240 | New Org: dynamic org from test-data/org.json</t>
         </is>
       </c>
     </row>
@@ -533,7 +566,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>tests/test1.spec.ts, tests/test2.spec.ts</t>
+          <t>tests/test1.spec.ts, tests/test2.spec.ts, tests/CreateOrganization.spec.ts, tests/Flow1-NewOrganization.spec.ts, tests/Flow2-NewOrganization.spec.ts</t>
         </is>
       </c>
     </row>
@@ -545,7 +578,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Flow 1 -&gt; Flow 2</t>
+          <t>Legacy: Flow 1 (test1) -&gt; Flow 2 (test2). New Org: Create Organization -&gt; Flow1-NewOrganization -&gt; Flow2-NewOrganization</t>
         </is>
       </c>
     </row>
@@ -557,7 +590,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Automated onboarding, rent collection, service request, vendor billing, tenant invoicing, and payment journeys</t>
+          <t>Automated organization registration, onboarding, rent collection, service request, vendor billing, tenant invoicing, and payment journeys for both existing (test240) and newly created organizations</t>
         </is>
       </c>
     </row>
@@ -570,26 +603,62 @@
       <c r="B12" s="3" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>TC-01</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Create property, onboard tenant, create rent invoice, tenant pays via Razorpay</t>
+          <t>Create property, onboard tenant, create rent invoice, tenant pays via Razorpay (org: test240)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>TC-02</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Tenant request -&gt; vendor -&gt; task -&gt; tenant approval -&gt; vendor bill paid -&gt; tenant service invoice paid</t>
+          <t>Tenant request -&gt; vendor -&gt; task -&gt; tenant approval -&gt; vendor bill paid -&gt; tenant service invoice paid (org: test240)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>TC-03</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Create new organization via registration + Stripe card verification; save credentials to org.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>TC-04</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>New-org Flow 1: configure Razorpay, create property, onboard tenant, rent invoice, Razorpay pay; save tenant-new-org.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>TC-05</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>New-org Flow 2: tenant request -&gt; vendor -&gt; task -&gt; approval -&gt; bill paid -&gt; service invoice paid (uses org.json + tenant-new-org.json)</t>
         </is>
       </c>
     </row>
@@ -2794,4 +2863,2939 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Create Organization - register new org and save login data</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Test ID</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>TC-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>End-to-end / Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>TEST environment is available; Stripe test card and referral code TEST9 are valid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Test ID</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Step #</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>Actor</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="45" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>TC-03</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Create Organization - register new org and save login data</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>Open https://test.propexcel.com/login</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>Welcome Back login page is displayed</t>
+        </is>
+      </c>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H9" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I9" s="10" t="inlineStr">
+        <is>
+          <t>TEST environment is available; Stripe test card and referral code TEST9 are valid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>TC-03</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>Create Organization - register new org and save login data</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>Click Create a new organization</t>
+        </is>
+      </c>
+      <c r="F10" s="10" t="inlineStr">
+        <is>
+          <t>Create Account page/step is displayed</t>
+        </is>
+      </c>
+      <c r="G10" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H10" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I10" s="10" t="n"/>
+    </row>
+    <row r="11" ht="45" customHeight="1">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>TC-03</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Create Organization - register new org and save login data</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>Enter Organization Name as Automation ###, Organization Code as automation-###, admin email as automation###@yopmail.com, password Test2026$, and referral code TEST9</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="inlineStr">
+        <is>
+          <t>Details fields are filled correctly</t>
+        </is>
+      </c>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H11" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I11" s="10" t="n"/>
+    </row>
+    <row r="12" ht="45" customHeight="1">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>TC-03</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Create Organization - register new org and save login data</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>Click Continue</t>
+        </is>
+      </c>
+      <c r="F12" s="10" t="inlineStr">
+        <is>
+          <t>Customize workspace settings step is displayed</t>
+        </is>
+      </c>
+      <c r="G12" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H12" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I12" s="10" t="n"/>
+    </row>
+    <row r="13" ht="45" customHeight="1">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>TC-03</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Create Organization - register new org and save login data</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E13" s="10" t="inlineStr">
+        <is>
+          <t>Enter Number of Offices and Number of Coworking Spaces (random 10-50)</t>
+        </is>
+      </c>
+      <c r="F13" s="10" t="inlineStr">
+        <is>
+          <t>Office and space counts are set</t>
+        </is>
+      </c>
+      <c r="G13" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H13" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I13" s="10" t="n"/>
+    </row>
+    <row r="14" ht="45" customHeight="1">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>TC-03</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>Create Organization - register new org and save login data</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E14" s="10" t="inlineStr">
+        <is>
+          <t>Check I agree to the Terms and Conditions</t>
+        </is>
+      </c>
+      <c r="F14" s="10" t="inlineStr">
+        <is>
+          <t>Terms checkbox is selected</t>
+        </is>
+      </c>
+      <c r="G14" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H14" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I14" s="10" t="n"/>
+    </row>
+    <row r="15" ht="45" customHeight="1">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>TC-03</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Create Organization - register new org and save login data</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E15" s="10" t="inlineStr">
+        <is>
+          <t>Click Proceed to Register</t>
+        </is>
+      </c>
+      <c r="F15" s="10" t="inlineStr">
+        <is>
+          <t>Stripe Subscribe / checkout page opens</t>
+        </is>
+      </c>
+      <c r="G15" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H15" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I15" s="10" t="n"/>
+    </row>
+    <row r="16" ht="45" customHeight="1">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>TC-03</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>Create Organization - register new org and save login data</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E16" s="10" t="inlineStr">
+        <is>
+          <t>Enter Stripe test card 4000003560000123, future expiry, CVC, and cardholder name = organization name</t>
+        </is>
+      </c>
+      <c r="F16" s="10" t="inlineStr">
+        <is>
+          <t>Card details are accepted in Stripe fields</t>
+        </is>
+      </c>
+      <c r="G16" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H16" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I16" s="10" t="n"/>
+    </row>
+    <row r="17" ht="45" customHeight="1">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>TC-03</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>Create Organization - register new org and save login data</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="D17" s="10" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E17" s="10" t="inlineStr">
+        <is>
+          <t>Click Subscribe</t>
+        </is>
+      </c>
+      <c r="F17" s="10" t="inlineStr">
+        <is>
+          <t>3D Secure challenge is displayed</t>
+        </is>
+      </c>
+      <c r="G17" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H17" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I17" s="10" t="n"/>
+    </row>
+    <row r="18" ht="45" customHeight="1">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>TC-03</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Create Organization - register new org and save login data</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
+        <is>
+          <t>Click COMPLETE on 3D Secure 2 Test Page (retry until challenge closes)</t>
+        </is>
+      </c>
+      <c r="F18" s="10" t="inlineStr">
+        <is>
+          <t>3DS challenge closes and payment processing completes</t>
+        </is>
+      </c>
+      <c r="G18" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H18" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I18" s="10" t="n"/>
+    </row>
+    <row r="19" ht="45" customHeight="1">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>TC-03</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>Create Organization - register new org and save login data</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E19" s="10" t="inlineStr">
+        <is>
+          <t>Wait for redirect to PropExcel login</t>
+        </is>
+      </c>
+      <c r="F19" s="10" t="inlineStr">
+        <is>
+          <t>Welcome Back page is displayed</t>
+        </is>
+      </c>
+      <c r="G19" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H19" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I19" s="10" t="n"/>
+    </row>
+    <row r="20" ht="45" customHeight="1">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>TC-03</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>Create Organization - register new org and save login data</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="E20" s="10" t="inlineStr">
+        <is>
+          <t>Save orgName, orgId, email, password, offices, spaces to test-data/org.json</t>
+        </is>
+      </c>
+      <c r="F20" s="10" t="inlineStr">
+        <is>
+          <t>org.json is available for Flow1-NewOrganization and Flow2-NewOrganization</t>
+        </is>
+      </c>
+      <c r="G20" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H20" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I20" s="10" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Test ID</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>TC-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>End-to-end / Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>TC-03 completed successfully and test-data/org.json exists with valid Super Admin credentials for the new organization.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Test ID</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Step #</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>Actor</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="45" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>TC-04</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>Login using orgId, email, and password from test-data/org.json</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>Dashboard/Properties area loads after leaving /login</t>
+        </is>
+      </c>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H9" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I9" s="10" t="inlineStr">
+        <is>
+          <t>TC-03 completed successfully and test-data/org.json exists with valid Super Admin credentials for the new organization.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>TC-04</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>Dismiss PropExcel End-to-End Flow tour (X/Escape) and Notifications modal if shown</t>
+        </is>
+      </c>
+      <c r="F10" s="10" t="inlineStr">
+        <is>
+          <t>Tour/notifications are closed and UI is usable</t>
+        </is>
+      </c>
+      <c r="G10" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H10" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I10" s="10" t="n"/>
+    </row>
+    <row r="11" ht="45" customHeight="1">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>TC-04</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>Open Admin module (top-nav gear) -&gt; Integrations -&gt; Razorpay; enter Key ID rzp_test_Strt5pbr1bvoIR and Key Secret; click Save Settings</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="inlineStr">
+        <is>
+          <t>Razorpay integration settings are saved</t>
+        </is>
+      </c>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H11" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I11" s="10" t="n"/>
+    </row>
+    <row r="12" ht="45" customHeight="1">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>TC-04</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>Open Property module (top-nav) -&gt; Properties</t>
+        </is>
+      </c>
+      <c r="F12" s="10" t="inlineStr">
+        <is>
+          <t>Properties page heading is displayed</t>
+        </is>
+      </c>
+      <c r="G12" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H12" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I12" s="10" t="n"/>
+    </row>
+    <row r="13" ht="45" customHeight="1">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>TC-04</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E13" s="10" t="inlineStr">
+        <is>
+          <t>Click + Create Property and create Office/Building with generated name, category, group, area, monthly rent, and tax</t>
+        </is>
+      </c>
+      <c r="F13" s="10" t="inlineStr">
+        <is>
+          <t>Property is created successfully</t>
+        </is>
+      </c>
+      <c r="G13" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H13" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I13" s="10" t="n"/>
+    </row>
+    <row r="14" ht="45" customHeight="1">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>TC-04</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E14" s="10" t="inlineStr">
+        <is>
+          <t>Go to CRM Contacts and create a new contact with generated tenant details</t>
+        </is>
+      </c>
+      <c r="F14" s="10" t="inlineStr">
+        <is>
+          <t>Contact appears in contacts list</t>
+        </is>
+      </c>
+      <c r="G14" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H14" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I14" s="10" t="n"/>
+    </row>
+    <row r="15" ht="45" customHeight="1">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>TC-04</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E15" s="10" t="inlineStr">
+        <is>
+          <t>Open contact and create lead</t>
+        </is>
+      </c>
+      <c r="F15" s="10" t="inlineStr">
+        <is>
+          <t>Lead is created successfully</t>
+        </is>
+      </c>
+      <c r="G15" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H15" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I15" s="10" t="n"/>
+    </row>
+    <row r="16" ht="45" customHeight="1">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>TC-04</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E16" s="10" t="inlineStr">
+        <is>
+          <t>Convert lead to deal and select payment type</t>
+        </is>
+      </c>
+      <c r="F16" s="10" t="inlineStr">
+        <is>
+          <t>Deal Details page opens</t>
+        </is>
+      </c>
+      <c r="G16" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H16" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I16" s="10" t="n"/>
+    </row>
+    <row r="17" ht="45" customHeight="1">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>TC-04</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="D17" s="10" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E17" s="10" t="inlineStr">
+        <is>
+          <t>Add created property to the deal and ensure tax is set</t>
+        </is>
+      </c>
+      <c r="F17" s="10" t="inlineStr">
+        <is>
+          <t>Property is attached to the deal</t>
+        </is>
+      </c>
+      <c r="G17" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H17" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I17" s="10" t="n"/>
+    </row>
+    <row r="18" ht="45" customHeight="1">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>TC-04</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
+        <is>
+          <t>Approve the deal</t>
+        </is>
+      </c>
+      <c r="F18" s="10" t="inlineStr">
+        <is>
+          <t>Deal is approved</t>
+        </is>
+      </c>
+      <c r="G18" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H18" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I18" s="10" t="n"/>
+    </row>
+    <row r="19" ht="45" customHeight="1">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>TC-04</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E19" s="10" t="inlineStr">
+        <is>
+          <t>Create/view contract and approve the contract</t>
+        </is>
+      </c>
+      <c r="F19" s="10" t="inlineStr">
+        <is>
+          <t>Contract is approved</t>
+        </is>
+      </c>
+      <c r="G19" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H19" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I19" s="10" t="n"/>
+    </row>
+    <row r="20" ht="45" customHeight="1">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>TC-04</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E20" s="10" t="inlineStr">
+        <is>
+          <t>Create tenant user from Action Buttons tab</t>
+        </is>
+      </c>
+      <c r="F20" s="10" t="inlineStr">
+        <is>
+          <t>Tenant user is created and password is captured from dialog or YOPmail</t>
+        </is>
+      </c>
+      <c r="G20" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H20" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I20" s="10" t="n"/>
+    </row>
+    <row r="21" ht="45" customHeight="1">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>TC-04</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="D21" s="10" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E21" s="10" t="inlineStr">
+        <is>
+          <t>Create move-in request with current move-in date</t>
+        </is>
+      </c>
+      <c r="F21" s="10" t="inlineStr">
+        <is>
+          <t>Move-in request is created</t>
+        </is>
+      </c>
+      <c r="G21" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H21" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I21" s="10" t="n"/>
+    </row>
+    <row r="22" ht="45" customHeight="1">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>TC-04</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="D22" s="10" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E22" s="10" t="inlineStr">
+        <is>
+          <t>Go to Operations Requests, open move-in request, start progress, complete request, and mark completed</t>
+        </is>
+      </c>
+      <c r="F22" s="10" t="inlineStr">
+        <is>
+          <t>Move-in request becomes completed</t>
+        </is>
+      </c>
+      <c r="G22" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H22" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I22" s="10" t="n"/>
+    </row>
+    <row r="23" ht="45" customHeight="1">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>TC-04</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="D23" s="10" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E23" s="10" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+      <c r="F23" s="10" t="inlineStr">
+        <is>
+          <t>Login page is displayed</t>
+        </is>
+      </c>
+      <c r="G23" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H23" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I23" s="10" t="n"/>
+    </row>
+    <row r="24" ht="45" customHeight="1">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>TC-04</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
+        </is>
+      </c>
+      <c r="C24" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="D24" s="10" t="inlineStr">
+        <is>
+          <t>Tenant</t>
+        </is>
+      </c>
+      <c r="E24" s="10" t="inlineStr">
+        <is>
+          <t>Login with generated tenant credentials (orgId from org.json) from YOPmail or captured password</t>
+        </is>
+      </c>
+      <c r="F24" s="10" t="inlineStr">
+        <is>
+          <t>Tenant portal opens successfully</t>
+        </is>
+      </c>
+      <c r="G24" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H24" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I24" s="10" t="n"/>
+    </row>
+    <row r="25" ht="45" customHeight="1">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>TC-04</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
+        </is>
+      </c>
+      <c r="C25" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="D25" s="10" t="inlineStr">
+        <is>
+          <t>Tenant</t>
+        </is>
+      </c>
+      <c r="E25" s="10" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+      <c r="F25" s="10" t="inlineStr">
+        <is>
+          <t>Login page is displayed</t>
+        </is>
+      </c>
+      <c r="G25" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H25" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I25" s="10" t="n"/>
+    </row>
+    <row r="26" ht="45" customHeight="1">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>TC-04</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
+        </is>
+      </c>
+      <c r="C26" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="D26" s="10" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E26" s="10" t="inlineStr">
+        <is>
+          <t>Login again using org.json credentials and navigate to Accounts Invoices</t>
+        </is>
+      </c>
+      <c r="F26" s="10" t="inlineStr">
+        <is>
+          <t>Invoices page is displayed</t>
+        </is>
+      </c>
+      <c r="G26" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H26" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I26" s="10" t="n"/>
+    </row>
+    <row r="27" ht="45" customHeight="1">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>TC-04</t>
+        </is>
+      </c>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="n">
+        <v>19</v>
+      </c>
+      <c r="D27" s="10" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E27" s="10" t="inlineStr">
+        <is>
+          <t>Create invoice for tenant and add line item using item rent, Chart of Account 4000 - Rental Income, amount 10000</t>
+        </is>
+      </c>
+      <c r="F27" s="10" t="inlineStr">
+        <is>
+          <t>Invoice draft is created</t>
+        </is>
+      </c>
+      <c r="G27" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H27" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I27" s="10" t="n"/>
+    </row>
+    <row r="28" ht="45" customHeight="1">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>TC-04</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
+        </is>
+      </c>
+      <c r="C28" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="D28" s="10" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E28" s="10" t="inlineStr">
+        <is>
+          <t>Submit/publish invoice</t>
+        </is>
+      </c>
+      <c r="F28" s="10" t="inlineStr">
+        <is>
+          <t>Invoice number is generated and invoice is due/visible to tenant</t>
+        </is>
+      </c>
+      <c r="G28" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H28" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I28" s="10" t="n"/>
+    </row>
+    <row r="29" ht="45" customHeight="1">
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t>TC-04</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="D29" s="10" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E29" s="10" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+      <c r="F29" s="10" t="inlineStr">
+        <is>
+          <t>Login page is displayed</t>
+        </is>
+      </c>
+      <c r="G29" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H29" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I29" s="10" t="n"/>
+    </row>
+    <row r="30" ht="45" customHeight="1">
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t>TC-04</t>
+        </is>
+      </c>
+      <c r="B30" s="10" t="inlineStr">
+        <is>
+          <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
+        </is>
+      </c>
+      <c r="C30" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="D30" s="10" t="inlineStr">
+        <is>
+          <t>Tenant</t>
+        </is>
+      </c>
+      <c r="E30" s="10" t="inlineStr">
+        <is>
+          <t>Login, open tenant invoices, open created invoice, click Pay Online and Pay with Razorpay</t>
+        </is>
+      </c>
+      <c r="F30" s="10" t="inlineStr">
+        <is>
+          <t>Razorpay checkout opens</t>
+        </is>
+      </c>
+      <c r="G30" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H30" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I30" s="10" t="n"/>
+    </row>
+    <row r="31" ht="45" customHeight="1">
+      <c r="A31" s="10" t="inlineStr">
+        <is>
+          <t>TC-04</t>
+        </is>
+      </c>
+      <c r="B31" s="10" t="inlineStr">
+        <is>
+          <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
+        </is>
+      </c>
+      <c r="C31" s="10" t="n">
+        <v>23</v>
+      </c>
+      <c r="D31" s="10" t="inlineStr">
+        <is>
+          <t>Tenant</t>
+        </is>
+      </c>
+      <c r="E31" s="10" t="inlineStr">
+        <is>
+          <t>Complete test payment using Netbanking -&gt; Bank of Baroda -&gt; Success</t>
+        </is>
+      </c>
+      <c r="F31" s="10" t="inlineStr">
+        <is>
+          <t>Invoice status becomes PAID</t>
+        </is>
+      </c>
+      <c r="G31" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H31" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I31" s="10" t="n"/>
+    </row>
+    <row r="32" ht="45" customHeight="1">
+      <c r="A32" s="10" t="inlineStr">
+        <is>
+          <t>TC-04</t>
+        </is>
+      </c>
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
+        </is>
+      </c>
+      <c r="C32" s="10" t="n">
+        <v>24</v>
+      </c>
+      <c r="D32" s="10" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="E32" s="10" t="inlineStr">
+        <is>
+          <t>Save tenant details to test-data/tenant-new-org.json for Flow 2 New Org reuse</t>
+        </is>
+      </c>
+      <c r="F32" s="10" t="inlineStr">
+        <is>
+          <t>tenant-new-org.json is available for Flow2-NewOrganization</t>
+        </is>
+      </c>
+      <c r="G32" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H32" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I32" s="10" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Flow 2 with New Organization - request, vendor bill, service invoice, and payment</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Test ID</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>TC-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>End-to-end / Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>TC-04 completed successfully; test-data/org.json and test-data/tenant-new-org.json exist with valid credentials.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Test ID</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Step #</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>Actor</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="45" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>TC-05</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Flow 2 with New Organization - request, vendor bill, service invoice, and payment</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>Tenant</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>Login using tenant credentials from tenant-new-org.json and orgId from org.json/tenant file</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>Tenant dashboard opens</t>
+        </is>
+      </c>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H9" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I9" s="10" t="inlineStr">
+        <is>
+          <t>TC-04 completed successfully; test-data/org.json and test-data/tenant-new-org.json exist with valid credentials.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>TC-05</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>Flow 2 with New Organization - request, vendor bill, service invoice, and payment</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>Tenant</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>Go to Requests and create a new request with property, title, shared category (Maintenance/Cleaning/Other), priority, and description</t>
+        </is>
+      </c>
+      <c r="F10" s="10" t="inlineStr">
+        <is>
+          <t>Request is submitted successfully</t>
+        </is>
+      </c>
+      <c r="G10" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H10" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I10" s="10" t="n"/>
+    </row>
+    <row r="11" ht="45" customHeight="1">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>TC-05</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Flow 2 with New Organization - request, vendor bill, service invoice, and payment</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>Tenant</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="inlineStr">
+        <is>
+          <t>Login page is displayed</t>
+        </is>
+      </c>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H11" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I11" s="10" t="n"/>
+    </row>
+    <row r="12" ht="45" customHeight="1">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>TC-05</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Flow 2 with New Organization - request, vendor bill, service invoice, and payment</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>Login using Super Admin credentials from org.json</t>
+        </is>
+      </c>
+      <c r="F12" s="10" t="inlineStr">
+        <is>
+          <t>Admin home page opens</t>
+        </is>
+      </c>
+      <c r="G12" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H12" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I12" s="10" t="n"/>
+    </row>
+    <row r="13" ht="45" customHeight="1">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>TC-05</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Flow 2 with New Organization - request, vendor bill, service invoice, and payment</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E13" s="10" t="inlineStr">
+        <is>
+          <t>Go to Accounts Vendors</t>
+        </is>
+      </c>
+      <c r="F13" s="10" t="inlineStr">
+        <is>
+          <t>Vendors page is displayed</t>
+        </is>
+      </c>
+      <c r="G13" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H13" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I13" s="10" t="n"/>
+    </row>
+    <row r="14" ht="45" customHeight="1">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>TC-05</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>Flow 2 with New Organization - request, vendor bill, service invoice, and payment</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E14" s="10" t="inlineStr">
+        <is>
+          <t>Create vendor using same shared category as tenant request and fill GST, contact, and address details</t>
+        </is>
+      </c>
+      <c r="F14" s="10" t="inlineStr">
+        <is>
+          <t>Vendor is created successfully</t>
+        </is>
+      </c>
+      <c r="G14" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H14" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I14" s="10" t="n"/>
+    </row>
+    <row r="15" ht="45" customHeight="1">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>TC-05</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Flow 2 with New Organization - request, vendor bill, service invoice, and payment</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E15" s="10" t="inlineStr">
+        <is>
+          <t>Go to Operations Requests and open the request created in this run</t>
+        </is>
+      </c>
+      <c r="F15" s="10" t="inlineStr">
+        <is>
+          <t>Request details page opens</t>
+        </is>
+      </c>
+      <c r="G15" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H15" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I15" s="10" t="n"/>
+    </row>
+    <row r="16" ht="45" customHeight="1">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>TC-05</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>Flow 2 with New Organization - request, vendor bill, service invoice, and payment</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E16" s="10" t="inlineStr">
+        <is>
+          <t>Click Start Progress</t>
+        </is>
+      </c>
+      <c r="F16" s="10" t="inlineStr">
+        <is>
+          <t>Request moves to In Progress</t>
+        </is>
+      </c>
+      <c r="G16" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H16" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I16" s="10" t="n"/>
+    </row>
+    <row r="17" ht="45" customHeight="1">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>TC-05</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>Flow 2 with New Organization - request, vendor bill, service invoice, and payment</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="D17" s="10" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E17" s="10" t="inlineStr">
+        <is>
+          <t>Add task with task title, status Open, random priority, and assign the created vendor</t>
+        </is>
+      </c>
+      <c r="F17" s="10" t="inlineStr">
+        <is>
+          <t>Task is created successfully</t>
+        </is>
+      </c>
+      <c r="G17" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H17" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I17" s="10" t="n"/>
+    </row>
+    <row r="18" ht="45" customHeight="1">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>TC-05</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Flow 2 with New Organization - request, vendor bill, service invoice, and payment</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
+        <is>
+          <t>Open task from Tasks page and change status from Open to Done</t>
+        </is>
+      </c>
+      <c r="F18" s="10" t="inlineStr">
+        <is>
+          <t>Task status becomes Done</t>
+        </is>
+      </c>
+      <c r="G18" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H18" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I18" s="10" t="n"/>
+    </row>
+    <row r="19" ht="45" customHeight="1">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>TC-05</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>Flow 2 with New Organization - request, vendor bill, service invoice, and payment</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E19" s="10" t="inlineStr">
+        <is>
+          <t>Return to Requests and click Request for Tenant Approval</t>
+        </is>
+      </c>
+      <c r="F19" s="10" t="inlineStr">
+        <is>
+          <t>Request moves to Tenant Approval Pending</t>
+        </is>
+      </c>
+      <c r="G19" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H19" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I19" s="10" t="n"/>
+    </row>
+    <row r="20" ht="45" customHeight="1">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>TC-05</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>Flow 2 with New Organization - request, vendor bill, service invoice, and payment</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E20" s="10" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+      <c r="F20" s="10" t="inlineStr">
+        <is>
+          <t>Login page is displayed</t>
+        </is>
+      </c>
+      <c r="G20" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H20" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I20" s="10" t="n"/>
+    </row>
+    <row r="21" ht="45" customHeight="1">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>TC-05</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>Flow 2 with New Organization - request, vendor bill, service invoice, and payment</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="D21" s="10" t="inlineStr">
+        <is>
+          <t>Tenant</t>
+        </is>
+      </c>
+      <c r="E21" s="10" t="inlineStr">
+        <is>
+          <t>Login again, open Requests from sidebar, and open the request in Tenant Approval Pending state</t>
+        </is>
+      </c>
+      <c r="F21" s="10" t="inlineStr">
+        <is>
+          <t>Pending request details page opens</t>
+        </is>
+      </c>
+      <c r="G21" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H21" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I21" s="10" t="n"/>
+    </row>
+    <row r="22" ht="45" customHeight="1">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>TC-05</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>Flow 2 with New Organization - request, vendor bill, service invoice, and payment</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="D22" s="10" t="inlineStr">
+        <is>
+          <t>Tenant</t>
+        </is>
+      </c>
+      <c r="E22" s="10" t="inlineStr">
+        <is>
+          <t>Click Approve Request</t>
+        </is>
+      </c>
+      <c r="F22" s="10" t="inlineStr">
+        <is>
+          <t>Request is approved/completed successfully</t>
+        </is>
+      </c>
+      <c r="G22" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H22" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I22" s="10" t="n"/>
+    </row>
+    <row r="23" ht="45" customHeight="1">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>TC-05</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>Flow 2 with New Organization - request, vendor bill, service invoice, and payment</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="D23" s="10" t="inlineStr">
+        <is>
+          <t>Tenant</t>
+        </is>
+      </c>
+      <c r="E23" s="10" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+      <c r="F23" s="10" t="inlineStr">
+        <is>
+          <t>Login page is displayed</t>
+        </is>
+      </c>
+      <c r="G23" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H23" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I23" s="10" t="n"/>
+    </row>
+    <row r="24" ht="45" customHeight="1">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>TC-05</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>Flow 2 with New Organization - request, vendor bill, service invoice, and payment</t>
+        </is>
+      </c>
+      <c r="C24" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="D24" s="10" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E24" s="10" t="inlineStr">
+        <is>
+          <t>Login again using org.json and go to Accounts Bills</t>
+        </is>
+      </c>
+      <c r="F24" s="10" t="inlineStr">
+        <is>
+          <t>Bills page is displayed</t>
+        </is>
+      </c>
+      <c r="G24" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H24" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I24" s="10" t="n"/>
+    </row>
+    <row r="25" ht="45" customHeight="1">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>TC-05</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>Flow 2 with New Organization - request, vendor bill, service invoice, and payment</t>
+        </is>
+      </c>
+      <c r="C25" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="D25" s="10" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E25" s="10" t="inlineStr">
+        <is>
+          <t>Create bill and fill reference number, vendor, tenant, related request, related task, and property</t>
+        </is>
+      </c>
+      <c r="F25" s="10" t="inlineStr">
+        <is>
+          <t>Bill draft form is filled correctly</t>
+        </is>
+      </c>
+      <c r="G25" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H25" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I25" s="10" t="n"/>
+    </row>
+    <row r="26" ht="45" customHeight="1">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>TC-05</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>Flow 2 with New Organization - request, vendor bill, service invoice, and payment</t>
+        </is>
+      </c>
+      <c r="C26" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="D26" s="10" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E26" s="10" t="inlineStr">
+        <is>
+          <t>Add bill line item using category-based item name, quantity 1-5, unit price, Chart of Account 4100 - Service Revenue, and GST</t>
+        </is>
+      </c>
+      <c r="F26" s="10" t="inlineStr">
+        <is>
+          <t>Bill line item is saved</t>
+        </is>
+      </c>
+      <c r="G26" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H26" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I26" s="10" t="n"/>
+    </row>
+    <row r="27" ht="45" customHeight="1">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>TC-05</t>
+        </is>
+      </c>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>Flow 2 with New Organization - request, vendor bill, service invoice, and payment</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="n">
+        <v>19</v>
+      </c>
+      <c r="D27" s="10" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E27" s="10" t="inlineStr">
+        <is>
+          <t>Submit bill</t>
+        </is>
+      </c>
+      <c r="F27" s="10" t="inlineStr">
+        <is>
+          <t>Bill status becomes Pending</t>
+        </is>
+      </c>
+      <c r="G27" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H27" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I27" s="10" t="n"/>
+    </row>
+    <row r="28" ht="45" customHeight="1">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>TC-05</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>Flow 2 with New Organization - request, vendor bill, service invoice, and payment</t>
+        </is>
+      </c>
+      <c r="C28" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="D28" s="10" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E28" s="10" t="inlineStr">
+        <is>
+          <t>Open pending bill and click Make Payment</t>
+        </is>
+      </c>
+      <c r="F28" s="10" t="inlineStr">
+        <is>
+          <t>Make Payment page/dialog opens</t>
+        </is>
+      </c>
+      <c r="G28" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H28" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I28" s="10" t="n"/>
+    </row>
+    <row r="29" ht="45" customHeight="1">
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t>TC-05</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>Flow 2 with New Organization - request, vendor bill, service invoice, and payment</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="D29" s="10" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E29" s="10" t="inlineStr">
+        <is>
+          <t>Select the bill, choose Chart of Account 4100 - Service Revenue, and confirm payment</t>
+        </is>
+      </c>
+      <c r="F29" s="10" t="inlineStr">
+        <is>
+          <t>Bill status becomes Paid</t>
+        </is>
+      </c>
+      <c r="G29" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H29" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I29" s="10" t="n"/>
+    </row>
+    <row r="30" ht="45" customHeight="1">
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t>TC-05</t>
+        </is>
+      </c>
+      <c r="B30" s="10" t="inlineStr">
+        <is>
+          <t>Flow 2 with New Organization - request, vendor bill, service invoice, and payment</t>
+        </is>
+      </c>
+      <c r="C30" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="D30" s="10" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E30" s="10" t="inlineStr">
+        <is>
+          <t>Go to Accounts Invoices and create invoice for the same tenant using Flow 2 item and amount</t>
+        </is>
+      </c>
+      <c r="F30" s="10" t="inlineStr">
+        <is>
+          <t>Invoice draft is created with Flow 2 values</t>
+        </is>
+      </c>
+      <c r="G30" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H30" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I30" s="10" t="n"/>
+    </row>
+    <row r="31" ht="45" customHeight="1">
+      <c r="A31" s="10" t="inlineStr">
+        <is>
+          <t>TC-05</t>
+        </is>
+      </c>
+      <c r="B31" s="10" t="inlineStr">
+        <is>
+          <t>Flow 2 with New Organization - request, vendor bill, service invoice, and payment</t>
+        </is>
+      </c>
+      <c r="C31" s="10" t="n">
+        <v>23</v>
+      </c>
+      <c r="D31" s="10" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E31" s="10" t="inlineStr">
+        <is>
+          <t>Submit/publish invoice</t>
+        </is>
+      </c>
+      <c r="F31" s="10" t="inlineStr">
+        <is>
+          <t>Invoice number is generated and invoice is visible to tenant</t>
+        </is>
+      </c>
+      <c r="G31" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H31" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I31" s="10" t="n"/>
+    </row>
+    <row r="32" ht="45" customHeight="1">
+      <c r="A32" s="10" t="inlineStr">
+        <is>
+          <t>TC-05</t>
+        </is>
+      </c>
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t>Flow 2 with New Organization - request, vendor bill, service invoice, and payment</t>
+        </is>
+      </c>
+      <c r="C32" s="10" t="n">
+        <v>24</v>
+      </c>
+      <c r="D32" s="10" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E32" s="10" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+      <c r="F32" s="10" t="inlineStr">
+        <is>
+          <t>Login page is displayed</t>
+        </is>
+      </c>
+      <c r="G32" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H32" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I32" s="10" t="n"/>
+    </row>
+    <row r="33" ht="45" customHeight="1">
+      <c r="A33" s="10" t="inlineStr">
+        <is>
+          <t>TC-05</t>
+        </is>
+      </c>
+      <c r="B33" s="10" t="inlineStr">
+        <is>
+          <t>Flow 2 with New Organization - request, vendor bill, service invoice, and payment</t>
+        </is>
+      </c>
+      <c r="C33" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="D33" s="10" t="inlineStr">
+        <is>
+          <t>Tenant</t>
+        </is>
+      </c>
+      <c r="E33" s="10" t="inlineStr">
+        <is>
+          <t>Login, go to tenant invoices, open created invoice, and click Pay Online / Pay with Razorpay</t>
+        </is>
+      </c>
+      <c r="F33" s="10" t="inlineStr">
+        <is>
+          <t>Razorpay checkout opens</t>
+        </is>
+      </c>
+      <c r="G33" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H33" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I33" s="10" t="n"/>
+    </row>
+    <row r="34" ht="45" customHeight="1">
+      <c r="A34" s="10" t="inlineStr">
+        <is>
+          <t>TC-05</t>
+        </is>
+      </c>
+      <c r="B34" s="10" t="inlineStr">
+        <is>
+          <t>Flow 2 with New Organization - request, vendor bill, service invoice, and payment</t>
+        </is>
+      </c>
+      <c r="C34" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="D34" s="10" t="inlineStr">
+        <is>
+          <t>Tenant</t>
+        </is>
+      </c>
+      <c r="E34" s="10" t="inlineStr">
+        <is>
+          <t>Complete test payment using Netbanking -&gt; Bank of Baroda -&gt; Success</t>
+        </is>
+      </c>
+      <c r="F34" s="10" t="inlineStr">
+        <is>
+          <t>Invoice status becomes PAID</t>
+        </is>
+      </c>
+      <c r="G34" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H34" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I34" s="10" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add new Playwright test files for CRM and enhance shared data utilities
- Introduced tests for creating contacts, leads, and deals in .
- Added tests for existing organization flows in  and .
- Implemented shared data utilities for managing CRM contacts and leads in .
- Updated  error messages for clarity on test execution requirements.
</commit_message>
<xml_diff>
--- a/PropExcel_Test_Cases.xlsx
+++ b/PropExcel_Test_Cases.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -510,6 +510,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -566,7 +567,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>tests/test1.spec.ts, tests/test2.spec.ts, tests/CreateOrganization.spec.ts, tests/Flow1-NewOrganization.spec.ts, tests/Flow2-NewOrganization.spec.ts</t>
+          <t>tests/Flow1-ExistingOrganization.spec.ts, tests/Flow2-ExistingOrganization.spec.ts, tests/CreateOrganization.spec.ts, tests/Flow1-NewOrganization.spec.ts, tests/Flow2-NewOrganization.spec.ts</t>
         </is>
       </c>
     </row>
@@ -578,7 +579,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Legacy: Flow 1 (test1) -&gt; Flow 2 (test2). New Org: Create Organization -&gt; Flow1-NewOrganization -&gt; Flow2-NewOrganization</t>
+          <t>Legacy: Flow 1 (Flow1-ExistingOrganization) -&gt; Flow 2 (Flow2-ExistingOrganization). New Org: Create Organization -&gt; Flow1-NewOrganization -&gt; Flow2-NewOrganization</t>
         </is>
       </c>
     </row>
@@ -594,6 +595,8 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
@@ -662,6 +665,9 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:B1"/>

</xml_diff>

<commit_message>
Update PropExcel_Test_Cases.xlsx with new test scenarios and data adjustments
</commit_message>
<xml_diff>
--- a/PropExcel_Test_Cases.xlsx
+++ b/PropExcel_Test_Cases.xlsx
@@ -13,8 +13,14 @@
     <sheet name="TC-03_CreateOrganization" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="TC-04_Flow1_NewOrg" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="TC-05_Flow2_NewOrg" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="TC-06_ContactsLeadsDeals" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="TC-07_ExistingContactPayment" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'TC-04_Flow1_NewOrg'!$A$8:$I$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'TC-06_ContactsLeadsDeals'!$A$8:$I$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'TC-07_ExistingContactPayment'!$A$8:$I$26</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -22,7 +28,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -46,6 +52,15 @@
       <color rgb="001F4E78"/>
       <sz val="14"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font/>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -65,7 +80,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -101,11 +116,12 @@
         <color rgb="00B0B0B0"/>
       </bottom>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -130,6 +146,25 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -496,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -510,7 +545,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -559,7 +593,7 @@
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="48" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Scripts</t>
@@ -567,11 +601,11 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>tests/Flow1-ExistingOrganization.spec.ts, tests/Flow2-ExistingOrganization.spec.ts, tests/CreateOrganization.spec.ts, tests/Flow1-NewOrganization.spec.ts, tests/Flow2-NewOrganization.spec.ts</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
+          <t>tests/Flow1-ExistingOrganization.spec.ts, tests/Flow2-ExistingOrganization.spec.ts, tests/CreateOrganization.spec.ts, tests/Flow1-NewOrganization.spec.ts, tests/Creating Contacts,Leads,Deals.spec.ts, tests/ExistingContact-ToTenantPayment.spec.ts, tests/Flow2-NewOrganization.spec.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Execution Order</t>
@@ -579,11 +613,11 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Legacy: Flow 1 (Flow1-ExistingOrganization) -&gt; Flow 2 (Flow2-ExistingOrganization). New Org: Create Organization -&gt; Flow1-NewOrganization -&gt; Flow2-NewOrganization</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
+          <t>Legacy: Flow 1 (Flow1-ExistingOrganization) -&gt; Flow 2 (Flow2-ExistingOrganization). New Org chain: Create Organization -&gt; Flow1-NewOrganization -&gt; Creating Contacts,Leads,Deals -&gt; ExistingContact-ToTenantPayment. Optional: Flow2-NewOrganization after Flow1 (uses tenant-new-org.json).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Purpose</t>
@@ -591,12 +625,10 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Automated organization registration, onboarding, rent collection, service request, vendor billing, tenant invoicing, and payment journeys for both existing (test240) and newly created organizations</t>
-        </is>
-      </c>
-    </row>
-    <row r="10"/>
-    <row r="11"/>
+          <t>Automated organization registration, CRM contacts/leads/deals, tenant onboarding, rent collection, service request, vendor billing, tenant invoicing, and Razorpay payment journeys for both existing (test240) and newly created organizations</t>
+        </is>
+      </c>
+    </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
@@ -605,69 +637,90 @@
       </c>
       <c r="B12" s="3" t="n"/>
     </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>TC-01</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Create property, onboard tenant, create rent invoice, tenant pays via Razorpay (org: test240)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>Create property, onboard tenant, create rent invoice, tenant pays via Razorpay (org: test240). Script: Flow1-ExistingOrganization.spec.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="32" customHeight="1">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>TC-02</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Tenant request -&gt; vendor -&gt; task -&gt; tenant approval -&gt; vendor bill paid -&gt; tenant service invoice paid (org: test240)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>Tenant request -&gt; vendor -&gt; task -&gt; tenant approval -&gt; vendor bill paid -&gt; tenant service invoice paid (org: test240). Script: Flow2-ExistingOrganization.spec.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="32" customHeight="1">
+      <c r="A15" s="13" t="inlineStr">
         <is>
           <t>TC-03</t>
         </is>
       </c>
-      <c r="B15" s="8" t="inlineStr">
-        <is>
-          <t>Create new organization via registration + Stripe card verification; save credentials to org.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="7" t="inlineStr">
+      <c r="B15" s="14" t="inlineStr">
+        <is>
+          <t>Create new organization via registration + Stripe card verification; save credentials to org.json. Script: CreateOrganization.spec.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="32" customHeight="1">
+      <c r="A16" s="13" t="inlineStr">
         <is>
           <t>TC-04</t>
         </is>
       </c>
-      <c r="B16" s="8" t="inlineStr">
-        <is>
-          <t>New-org Flow 1: configure Razorpay, create property, onboard tenant, rent invoice, Razorpay pay; save tenant-new-org.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="7" t="inlineStr">
+      <c r="B16" s="14" t="inlineStr">
+        <is>
+          <t>New-org Flow 1: Razorpay, GST 18% tax, Deal Approve workflow, create property, onboard tenant, rent invoice, Razorpay pay; save tenant-new-org.json. Script: Flow1-NewOrganization.spec.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="32" customHeight="1">
+      <c r="A17" s="13" t="inlineStr">
         <is>
           <t>TC-05</t>
         </is>
       </c>
-      <c r="B17" s="8" t="inlineStr">
-        <is>
-          <t>New-org Flow 2: tenant request -&gt; vendor -&gt; task -&gt; approval -&gt; bill paid -&gt; service invoice paid (uses org.json + tenant-new-org.json)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>New-org Flow 2: tenant request -&gt; vendor -&gt; task -&gt; approval -&gt; bill paid -&gt; service invoice paid (uses org.json + tenant-new-org.json). Script: Flow2-NewOrganization.spec.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="32" customHeight="1">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>TC-06</t>
+        </is>
+      </c>
+      <c r="B18" s="14" t="inlineStr">
+        <is>
+          <t>Create 4 contacts and 4 leads (separate random data); convert each lead to a deal; save crm-contacts-leads.json. Script: Creating Contacts,Leads,Deals.spec.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="32" customHeight="1">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>TC-07</t>
+        </is>
+      </c>
+      <c r="B19" s="14" t="inlineStr">
+        <is>
+          <t>Existing CRM contact -&gt; lead/deal -&gt; Vacant property -&gt; GST 18% pricing -&gt; approval workflow -&gt; tenant -&gt; rent invoice paid. Script: ExistingContact-ToTenantPayment.spec.ts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:B1"/>
@@ -3474,7 +3527,7 @@
       </c>
       <c r="F20" s="10" t="inlineStr">
         <is>
-          <t>org.json is available for Flow1-NewOrganization and Flow2-NewOrganization</t>
+          <t>org.json is available for Flow1-NewOrganization, Creating Contacts,Leads,Deals, ExistingContact-ToTenantPayment, and Flow2-NewOrganization</t>
         </is>
       </c>
       <c r="G20" s="10" t="inlineStr">
@@ -3498,9 +3551,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:I33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3515,59 +3568,117 @@
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
         </is>
       </c>
+      <c r="B1" s="16" t="n"/>
+      <c r="C1" s="16" t="n"/>
+      <c r="D1" s="16" t="n"/>
+      <c r="E1" s="16" t="n"/>
+      <c r="F1" s="16" t="n"/>
+      <c r="G1" s="16" t="n"/>
+      <c r="H1" s="16" t="n"/>
+      <c r="I1" s="16" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="16" t="n"/>
+      <c r="B2" s="16" t="n"/>
+      <c r="C2" s="16" t="n"/>
+      <c r="D2" s="16" t="n"/>
+      <c r="E2" s="16" t="n"/>
+      <c r="F2" s="16" t="n"/>
+      <c r="G2" s="16" t="n"/>
+      <c r="H2" s="16" t="n"/>
+      <c r="I2" s="16" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="17" t="inlineStr">
         <is>
           <t>Test ID</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="16" t="inlineStr">
         <is>
           <t>TC-04</t>
         </is>
       </c>
+      <c r="C3" s="16" t="n"/>
+      <c r="D3" s="16" t="n"/>
+      <c r="E3" s="16" t="n"/>
+      <c r="F3" s="16" t="n"/>
+      <c r="G3" s="16" t="n"/>
+      <c r="H3" s="16" t="n"/>
+      <c r="I3" s="16" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="n"/>
+      <c r="D4" s="16" t="n"/>
+      <c r="E4" s="16" t="n"/>
+      <c r="F4" s="16" t="n"/>
+      <c r="G4" s="16" t="n"/>
+      <c r="H4" s="16" t="n"/>
+      <c r="I4" s="16" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>End-to-end / Regression</t>
         </is>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="C5" s="16" t="n"/>
+      <c r="D5" s="16" t="n"/>
+      <c r="E5" s="16" t="n"/>
+      <c r="F5" s="16" t="n"/>
+      <c r="G5" s="16" t="n"/>
+      <c r="H5" s="16" t="n"/>
+      <c r="I5" s="16" t="n"/>
+    </row>
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>Precondition</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>TC-03 completed successfully and test-data/org.json exists with valid Super Admin credentials for the new organization.</t>
         </is>
       </c>
+      <c r="C6" s="16" t="n"/>
+      <c r="D6" s="16" t="n"/>
+      <c r="E6" s="16" t="n"/>
+      <c r="F6" s="16" t="n"/>
+      <c r="G6" s="16" t="n"/>
+      <c r="H6" s="16" t="n"/>
+      <c r="I6" s="16" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="16" t="n"/>
+      <c r="B7" s="16" t="n"/>
+      <c r="C7" s="16" t="n"/>
+      <c r="D7" s="16" t="n"/>
+      <c r="E7" s="16" t="n"/>
+      <c r="F7" s="16" t="n"/>
+      <c r="G7" s="16" t="n"/>
+      <c r="H7" s="16" t="n"/>
+      <c r="I7" s="16" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
@@ -3617,995 +3728,1038 @@
       </c>
     </row>
     <row r="9" ht="45" customHeight="1">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>TC-04</t>
         </is>
       </c>
-      <c r="B9" s="10" t="inlineStr">
+      <c r="B9" s="19" t="inlineStr">
         <is>
           <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
         </is>
       </c>
-      <c r="C9" s="10" t="n">
+      <c r="C9" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="D9" s="10" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E9" s="10" t="inlineStr">
+      <c r="D9" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E9" s="19" t="inlineStr">
         <is>
           <t>Login using orgId, email, and password from test-data/org.json</t>
         </is>
       </c>
-      <c r="F9" s="10" t="inlineStr">
+      <c r="F9" s="19" t="inlineStr">
         <is>
           <t>Dashboard/Properties area loads after leaving /login</t>
         </is>
       </c>
-      <c r="G9" s="10" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H9" s="10" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I9" s="10" t="inlineStr">
+      <c r="G9" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H9" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I9" s="19" t="inlineStr">
         <is>
           <t>TC-03 completed successfully and test-data/org.json exists with valid Super Admin credentials for the new organization.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="45" customHeight="1">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>TC-04</t>
         </is>
       </c>
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="19" t="inlineStr">
         <is>
           <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
         </is>
       </c>
-      <c r="C10" s="10" t="n">
+      <c r="C10" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="D10" s="10" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E10" s="10" t="inlineStr">
+      <c r="D10" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E10" s="19" t="inlineStr">
         <is>
           <t>Dismiss PropExcel End-to-End Flow tour (X/Escape) and Notifications modal if shown</t>
         </is>
       </c>
-      <c r="F10" s="10" t="inlineStr">
+      <c r="F10" s="19" t="inlineStr">
         <is>
           <t>Tour/notifications are closed and UI is usable</t>
         </is>
       </c>
-      <c r="G10" s="10" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H10" s="10" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I10" s="10" t="n"/>
+      <c r="G10" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H10" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I10" s="19" t="n"/>
     </row>
     <row r="11" ht="45" customHeight="1">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>TC-04</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="19" t="inlineStr">
         <is>
           <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
         </is>
       </c>
-      <c r="C11" s="10" t="n">
+      <c r="C11" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="D11" s="10" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E11" s="10" t="inlineStr">
+      <c r="D11" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E11" s="19" t="inlineStr">
         <is>
           <t>Open Admin module (top-nav gear) -&gt; Integrations -&gt; Razorpay; enter Key ID rzp_test_Strt5pbr1bvoIR and Key Secret; click Save Settings</t>
         </is>
       </c>
-      <c r="F11" s="10" t="inlineStr">
+      <c r="F11" s="19" t="inlineStr">
         <is>
           <t>Razorpay integration settings are saved</t>
         </is>
       </c>
-      <c r="G11" s="10" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H11" s="10" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I11" s="10" t="n"/>
+      <c r="G11" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H11" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I11" s="19" t="n"/>
     </row>
     <row r="12" ht="45" customHeight="1">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>TC-04</t>
         </is>
       </c>
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B12" s="19" t="inlineStr">
         <is>
           <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
         </is>
       </c>
-      <c r="C12" s="10" t="n">
+      <c r="C12" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="D12" s="10" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E12" s="10" t="inlineStr">
-        <is>
-          <t>Open Property module (top-nav) -&gt; Properties</t>
-        </is>
-      </c>
-      <c r="F12" s="10" t="inlineStr">
-        <is>
-          <t>Properties page heading is displayed</t>
-        </is>
-      </c>
-      <c r="G12" s="10" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H12" s="10" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I12" s="10" t="n"/>
+      <c r="D12" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E12" s="19" t="inlineStr">
+        <is>
+          <t>Open Accounts -&gt; Account Settings -&gt; Taxes. If VAT exists, delete it. If GST (18%) / GST-18 already exists, skip create; otherwise create tax name GST (18%), code GST-18, percentage 18</t>
+        </is>
+      </c>
+      <c r="F12" s="19" t="inlineStr">
+        <is>
+          <t>GST (18%) is the configured tax (VAT default is not used)</t>
+        </is>
+      </c>
+      <c r="G12" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H12" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I12" s="19" t="n"/>
     </row>
     <row r="13" ht="45" customHeight="1">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="19" t="inlineStr">
         <is>
           <t>TC-04</t>
         </is>
       </c>
-      <c r="B13" s="10" t="inlineStr">
+      <c r="B13" s="19" t="inlineStr">
         <is>
           <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
         </is>
       </c>
-      <c r="C13" s="10" t="n">
+      <c r="C13" s="19" t="n">
         <v>5</v>
       </c>
-      <c r="D13" s="10" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E13" s="10" t="inlineStr">
-        <is>
-          <t>Click + Create Property and create Office/Building with generated name, category, group, area, monthly rent, and tax</t>
-        </is>
-      </c>
-      <c r="F13" s="10" t="inlineStr">
-        <is>
-          <t>Property is created successfully</t>
-        </is>
-      </c>
-      <c r="G13" s="10" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H13" s="10" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I13" s="10" t="n"/>
+      <c r="D13" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E13" s="19" t="inlineStr">
+        <is>
+          <t>Open Admin -&gt; Approval Workflows. If Deal Approve already exists, skip. Else Create New Workflow, stay on Visual, click + Create Step, set Step Name Internal Approval, Approver Type User (Employee), select Super Admin, click Add Step (do not press Escape). Set Module CRM, Feature deals, Workflow Name Deal Approve, enable workflow, Save Changes</t>
+        </is>
+      </c>
+      <c r="F13" s="19" t="inlineStr">
+        <is>
+          <t>Deal Approve workflow is saved for CRM / deals</t>
+        </is>
+      </c>
+      <c r="G13" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H13" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I13" s="19" t="n"/>
     </row>
     <row r="14" ht="45" customHeight="1">
-      <c r="A14" s="10" t="inlineStr">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>TC-04</t>
         </is>
       </c>
-      <c r="B14" s="10" t="inlineStr">
+      <c r="B14" s="19" t="inlineStr">
         <is>
           <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
         </is>
       </c>
-      <c r="C14" s="10" t="n">
+      <c r="C14" s="19" t="n">
         <v>6</v>
       </c>
-      <c r="D14" s="10" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E14" s="10" t="inlineStr">
+      <c r="D14" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E14" s="19" t="inlineStr">
+        <is>
+          <t>Open Property module -&gt; Properties. Click + Create Property and create Office/Building with generated name, category, group, area, monthly rent, and Select Tax GST (18%)</t>
+        </is>
+      </c>
+      <c r="F14" s="19" t="inlineStr">
+        <is>
+          <t>Property is created successfully with GST 18%</t>
+        </is>
+      </c>
+      <c r="G14" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H14" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I14" s="19" t="n"/>
+    </row>
+    <row r="15" ht="45" customHeight="1">
+      <c r="A15" s="19" t="inlineStr">
+        <is>
+          <t>TC-04</t>
+        </is>
+      </c>
+      <c r="B15" s="19" t="inlineStr">
+        <is>
+          <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
+        </is>
+      </c>
+      <c r="C15" s="19" t="n">
+        <v>7</v>
+      </c>
+      <c r="D15" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E15" s="19" t="inlineStr">
         <is>
           <t>Go to CRM Contacts and create a new contact with generated tenant details</t>
         </is>
       </c>
-      <c r="F14" s="10" t="inlineStr">
+      <c r="F15" s="19" t="inlineStr">
         <is>
           <t>Contact appears in contacts list</t>
         </is>
       </c>
-      <c r="G14" s="10" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H14" s="10" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I14" s="10" t="n"/>
-    </row>
-    <row r="15" ht="45" customHeight="1">
-      <c r="A15" s="10" t="inlineStr">
+      <c r="G15" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H15" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I15" s="19" t="n"/>
+    </row>
+    <row r="16" ht="45" customHeight="1">
+      <c r="A16" s="19" t="inlineStr">
         <is>
           <t>TC-04</t>
         </is>
       </c>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B16" s="19" t="inlineStr">
         <is>
           <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
         </is>
       </c>
-      <c r="C15" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="D15" s="10" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E15" s="10" t="inlineStr">
+      <c r="C16" s="19" t="n">
+        <v>8</v>
+      </c>
+      <c r="D16" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E16" s="19" t="inlineStr">
         <is>
           <t>Open contact and create lead</t>
         </is>
       </c>
-      <c r="F15" s="10" t="inlineStr">
+      <c r="F16" s="19" t="inlineStr">
         <is>
           <t>Lead is created successfully</t>
         </is>
       </c>
-      <c r="G15" s="10" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H15" s="10" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I15" s="10" t="n"/>
-    </row>
-    <row r="16" ht="45" customHeight="1">
-      <c r="A16" s="10" t="inlineStr">
+      <c r="G16" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H16" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I16" s="19" t="n"/>
+    </row>
+    <row r="17" ht="45" customHeight="1">
+      <c r="A17" s="19" t="inlineStr">
         <is>
           <t>TC-04</t>
         </is>
       </c>
-      <c r="B16" s="10" t="inlineStr">
+      <c r="B17" s="19" t="inlineStr">
         <is>
           <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
         </is>
       </c>
-      <c r="C16" s="10" t="n">
-        <v>8</v>
-      </c>
-      <c r="D16" s="10" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E16" s="10" t="inlineStr">
+      <c r="C17" s="19" t="n">
+        <v>9</v>
+      </c>
+      <c r="D17" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E17" s="19" t="inlineStr">
         <is>
           <t>Convert lead to deal and select payment type</t>
         </is>
       </c>
-      <c r="F16" s="10" t="inlineStr">
+      <c r="F17" s="19" t="inlineStr">
         <is>
           <t>Deal Details page opens</t>
         </is>
       </c>
-      <c r="G16" s="10" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H16" s="10" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I16" s="10" t="n"/>
-    </row>
-    <row r="17" ht="45" customHeight="1">
-      <c r="A17" s="10" t="inlineStr">
+      <c r="G17" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H17" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I17" s="19" t="n"/>
+    </row>
+    <row r="18" ht="45" customHeight="1">
+      <c r="A18" s="19" t="inlineStr">
         <is>
           <t>TC-04</t>
         </is>
       </c>
-      <c r="B17" s="10" t="inlineStr">
+      <c r="B18" s="19" t="inlineStr">
         <is>
           <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
         </is>
       </c>
-      <c r="C17" s="10" t="n">
-        <v>9</v>
-      </c>
-      <c r="D17" s="10" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E17" s="10" t="inlineStr">
-        <is>
-          <t>Add created property to the deal and ensure tax is set</t>
-        </is>
-      </c>
-      <c r="F17" s="10" t="inlineStr">
-        <is>
-          <t>Property is attached to the deal</t>
-        </is>
-      </c>
-      <c r="G17" s="10" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H17" s="10" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I17" s="10" t="n"/>
-    </row>
-    <row r="18" ht="45" customHeight="1">
-      <c r="A18" s="10" t="inlineStr">
+      <c r="C18" s="19" t="n">
+        <v>10</v>
+      </c>
+      <c r="D18" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E18" s="19" t="inlineStr">
+        <is>
+          <t>Add created property to the deal and set tax to GST (18%) if needed; Save</t>
+        </is>
+      </c>
+      <c r="F18" s="19" t="inlineStr">
+        <is>
+          <t>Property is attached to the deal with GST 18%</t>
+        </is>
+      </c>
+      <c r="G18" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H18" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I18" s="19" t="n"/>
+    </row>
+    <row r="19" ht="45" customHeight="1">
+      <c r="A19" s="19" t="inlineStr">
         <is>
           <t>TC-04</t>
         </is>
       </c>
-      <c r="B18" s="10" t="inlineStr">
+      <c r="B19" s="19" t="inlineStr">
         <is>
           <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
         </is>
       </c>
-      <c r="C18" s="10" t="n">
-        <v>10</v>
-      </c>
-      <c r="D18" s="10" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E18" s="10" t="inlineStr">
-        <is>
-          <t>Approve the deal</t>
-        </is>
-      </c>
-      <c r="F18" s="10" t="inlineStr">
-        <is>
-          <t>Deal is approved</t>
-        </is>
-      </c>
-      <c r="G18" s="10" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H18" s="10" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I18" s="10" t="n"/>
-    </row>
-    <row r="19" ht="45" customHeight="1">
-      <c r="A19" s="10" t="inlineStr">
+      <c r="C19" s="19" t="n">
+        <v>11</v>
+      </c>
+      <c r="D19" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E19" s="19" t="inlineStr">
+        <is>
+          <t>Mark site visit done if required, click Submit for Approval, then Approve on Internal Approval and Confirm</t>
+        </is>
+      </c>
+      <c r="F19" s="19" t="inlineStr">
+        <is>
+          <t>Deal approval workflow completes (Create Contract / View Contract available)</t>
+        </is>
+      </c>
+      <c r="G19" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H19" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I19" s="19" t="n"/>
+    </row>
+    <row r="20" ht="45" customHeight="1">
+      <c r="A20" s="19" t="inlineStr">
         <is>
           <t>TC-04</t>
         </is>
       </c>
-      <c r="B19" s="10" t="inlineStr">
+      <c r="B20" s="19" t="inlineStr">
         <is>
           <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
         </is>
       </c>
-      <c r="C19" s="10" t="n">
-        <v>11</v>
-      </c>
-      <c r="D19" s="10" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E19" s="10" t="inlineStr">
+      <c r="C20" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="D20" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E20" s="19" t="inlineStr">
         <is>
           <t>Create/view contract and approve the contract</t>
         </is>
       </c>
-      <c r="F19" s="10" t="inlineStr">
+      <c r="F20" s="19" t="inlineStr">
         <is>
           <t>Contract is approved</t>
         </is>
       </c>
-      <c r="G19" s="10" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H19" s="10" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I19" s="10" t="n"/>
-    </row>
-    <row r="20" ht="45" customHeight="1">
-      <c r="A20" s="10" t="inlineStr">
+      <c r="G20" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H20" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I20" s="19" t="n"/>
+    </row>
+    <row r="21" ht="45" customHeight="1">
+      <c r="A21" s="19" t="inlineStr">
         <is>
           <t>TC-04</t>
         </is>
       </c>
-      <c r="B20" s="10" t="inlineStr">
+      <c r="B21" s="19" t="inlineStr">
         <is>
           <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
         </is>
       </c>
-      <c r="C20" s="10" t="n">
-        <v>12</v>
-      </c>
-      <c r="D20" s="10" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E20" s="10" t="inlineStr">
+      <c r="C21" s="19" t="n">
+        <v>13</v>
+      </c>
+      <c r="D21" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E21" s="19" t="inlineStr">
         <is>
           <t>Create tenant user from Action Buttons tab</t>
         </is>
       </c>
-      <c r="F20" s="10" t="inlineStr">
+      <c r="F21" s="19" t="inlineStr">
         <is>
           <t>Tenant user is created and password is captured from dialog or YOPmail</t>
         </is>
       </c>
-      <c r="G20" s="10" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H20" s="10" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I20" s="10" t="n"/>
-    </row>
-    <row r="21" ht="45" customHeight="1">
-      <c r="A21" s="10" t="inlineStr">
+      <c r="G21" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H21" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I21" s="19" t="n"/>
+    </row>
+    <row r="22" ht="45" customHeight="1">
+      <c r="A22" s="19" t="inlineStr">
         <is>
           <t>TC-04</t>
         </is>
       </c>
-      <c r="B21" s="10" t="inlineStr">
+      <c r="B22" s="19" t="inlineStr">
         <is>
           <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
         </is>
       </c>
-      <c r="C21" s="10" t="n">
-        <v>13</v>
-      </c>
-      <c r="D21" s="10" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E21" s="10" t="inlineStr">
+      <c r="C22" s="19" t="n">
+        <v>14</v>
+      </c>
+      <c r="D22" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E22" s="19" t="inlineStr">
         <is>
           <t>Create move-in request with current move-in date</t>
         </is>
       </c>
-      <c r="F21" s="10" t="inlineStr">
+      <c r="F22" s="19" t="inlineStr">
         <is>
           <t>Move-in request is created</t>
         </is>
       </c>
-      <c r="G21" s="10" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H21" s="10" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I21" s="10" t="n"/>
-    </row>
-    <row r="22" ht="45" customHeight="1">
-      <c r="A22" s="10" t="inlineStr">
+      <c r="G22" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H22" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I22" s="19" t="n"/>
+    </row>
+    <row r="23" ht="45" customHeight="1">
+      <c r="A23" s="19" t="inlineStr">
         <is>
           <t>TC-04</t>
         </is>
       </c>
-      <c r="B22" s="10" t="inlineStr">
+      <c r="B23" s="19" t="inlineStr">
         <is>
           <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
         </is>
       </c>
-      <c r="C22" s="10" t="n">
-        <v>14</v>
-      </c>
-      <c r="D22" s="10" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E22" s="10" t="inlineStr">
+      <c r="C23" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="D23" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E23" s="19" t="inlineStr">
         <is>
           <t>Go to Operations Requests, open move-in request, start progress, complete request, and mark completed</t>
         </is>
       </c>
-      <c r="F22" s="10" t="inlineStr">
+      <c r="F23" s="19" t="inlineStr">
         <is>
           <t>Move-in request becomes completed</t>
         </is>
       </c>
-      <c r="G22" s="10" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H22" s="10" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I22" s="10" t="n"/>
-    </row>
-    <row r="23" ht="45" customHeight="1">
-      <c r="A23" s="10" t="inlineStr">
+      <c r="G23" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H23" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I23" s="19" t="n"/>
+    </row>
+    <row r="24" ht="45" customHeight="1">
+      <c r="A24" s="19" t="inlineStr">
         <is>
           <t>TC-04</t>
         </is>
       </c>
-      <c r="B23" s="10" t="inlineStr">
+      <c r="B24" s="19" t="inlineStr">
         <is>
           <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
         </is>
       </c>
-      <c r="C23" s="10" t="n">
-        <v>15</v>
-      </c>
-      <c r="D23" s="10" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E23" s="10" t="inlineStr">
+      <c r="C24" s="19" t="n">
+        <v>16</v>
+      </c>
+      <c r="D24" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E24" s="19" t="inlineStr">
         <is>
           <t>Logout</t>
         </is>
       </c>
-      <c r="F23" s="10" t="inlineStr">
+      <c r="F24" s="19" t="inlineStr">
         <is>
           <t>Login page is displayed</t>
         </is>
       </c>
-      <c r="G23" s="10" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H23" s="10" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I23" s="10" t="n"/>
-    </row>
-    <row r="24" ht="45" customHeight="1">
-      <c r="A24" s="10" t="inlineStr">
+      <c r="G24" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H24" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I24" s="19" t="n"/>
+    </row>
+    <row r="25" ht="45" customHeight="1">
+      <c r="A25" s="19" t="inlineStr">
         <is>
           <t>TC-04</t>
         </is>
       </c>
-      <c r="B24" s="10" t="inlineStr">
+      <c r="B25" s="19" t="inlineStr">
         <is>
           <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
         </is>
       </c>
-      <c r="C24" s="10" t="n">
-        <v>16</v>
-      </c>
-      <c r="D24" s="10" t="inlineStr">
+      <c r="C25" s="19" t="n">
+        <v>17</v>
+      </c>
+      <c r="D25" s="19" t="inlineStr">
         <is>
           <t>Tenant</t>
         </is>
       </c>
-      <c r="E24" s="10" t="inlineStr">
+      <c r="E25" s="19" t="inlineStr">
         <is>
           <t>Login with generated tenant credentials (orgId from org.json) from YOPmail or captured password</t>
         </is>
       </c>
-      <c r="F24" s="10" t="inlineStr">
+      <c r="F25" s="19" t="inlineStr">
         <is>
           <t>Tenant portal opens successfully</t>
         </is>
       </c>
-      <c r="G24" s="10" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H24" s="10" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I24" s="10" t="n"/>
-    </row>
-    <row r="25" ht="45" customHeight="1">
-      <c r="A25" s="10" t="inlineStr">
+      <c r="G25" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H25" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I25" s="19" t="n"/>
+    </row>
+    <row r="26" ht="45" customHeight="1">
+      <c r="A26" s="19" t="inlineStr">
         <is>
           <t>TC-04</t>
         </is>
       </c>
-      <c r="B25" s="10" t="inlineStr">
+      <c r="B26" s="19" t="inlineStr">
         <is>
           <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
         </is>
       </c>
-      <c r="C25" s="10" t="n">
-        <v>17</v>
-      </c>
-      <c r="D25" s="10" t="inlineStr">
+      <c r="C26" s="19" t="n">
+        <v>18</v>
+      </c>
+      <c r="D26" s="19" t="inlineStr">
         <is>
           <t>Tenant</t>
         </is>
       </c>
-      <c r="E25" s="10" t="inlineStr">
+      <c r="E26" s="19" t="inlineStr">
         <is>
           <t>Logout</t>
         </is>
       </c>
-      <c r="F25" s="10" t="inlineStr">
+      <c r="F26" s="19" t="inlineStr">
         <is>
           <t>Login page is displayed</t>
         </is>
       </c>
-      <c r="G25" s="10" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H25" s="10" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I25" s="10" t="n"/>
-    </row>
-    <row r="26" ht="45" customHeight="1">
-      <c r="A26" s="10" t="inlineStr">
+      <c r="G26" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H26" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I26" s="19" t="n"/>
+    </row>
+    <row r="27" ht="45" customHeight="1">
+      <c r="A27" s="19" t="inlineStr">
         <is>
           <t>TC-04</t>
         </is>
       </c>
-      <c r="B26" s="10" t="inlineStr">
+      <c r="B27" s="19" t="inlineStr">
         <is>
           <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
         </is>
       </c>
-      <c r="C26" s="10" t="n">
-        <v>18</v>
-      </c>
-      <c r="D26" s="10" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E26" s="10" t="inlineStr">
+      <c r="C27" s="19" t="n">
+        <v>19</v>
+      </c>
+      <c r="D27" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E27" s="19" t="inlineStr">
         <is>
           <t>Login again using org.json credentials and navigate to Accounts Invoices</t>
         </is>
       </c>
-      <c r="F26" s="10" t="inlineStr">
+      <c r="F27" s="19" t="inlineStr">
         <is>
           <t>Invoices page is displayed</t>
         </is>
       </c>
-      <c r="G26" s="10" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H26" s="10" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I26" s="10" t="n"/>
-    </row>
-    <row r="27" ht="45" customHeight="1">
-      <c r="A27" s="10" t="inlineStr">
+      <c r="G27" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H27" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I27" s="19" t="n"/>
+    </row>
+    <row r="28" ht="45" customHeight="1">
+      <c r="A28" s="19" t="inlineStr">
         <is>
           <t>TC-04</t>
         </is>
       </c>
-      <c r="B27" s="10" t="inlineStr">
+      <c r="B28" s="19" t="inlineStr">
         <is>
           <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
         </is>
       </c>
-      <c r="C27" s="10" t="n">
-        <v>19</v>
-      </c>
-      <c r="D27" s="10" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E27" s="10" t="inlineStr">
+      <c r="C28" s="19" t="n">
+        <v>20</v>
+      </c>
+      <c r="D28" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E28" s="19" t="inlineStr">
         <is>
           <t>Create invoice for tenant and add line item using item rent, Chart of Account 4000 - Rental Income, amount 10000</t>
         </is>
       </c>
-      <c r="F27" s="10" t="inlineStr">
+      <c r="F28" s="19" t="inlineStr">
         <is>
           <t>Invoice draft is created</t>
         </is>
       </c>
-      <c r="G27" s="10" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H27" s="10" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I27" s="10" t="n"/>
-    </row>
-    <row r="28" ht="45" customHeight="1">
-      <c r="A28" s="10" t="inlineStr">
+      <c r="G28" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H28" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I28" s="19" t="n"/>
+    </row>
+    <row r="29" ht="45" customHeight="1">
+      <c r="A29" s="19" t="inlineStr">
         <is>
           <t>TC-04</t>
         </is>
       </c>
-      <c r="B28" s="10" t="inlineStr">
+      <c r="B29" s="19" t="inlineStr">
         <is>
           <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
         </is>
       </c>
-      <c r="C28" s="10" t="n">
-        <v>20</v>
-      </c>
-      <c r="D28" s="10" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E28" s="10" t="inlineStr">
+      <c r="C29" s="19" t="n">
+        <v>21</v>
+      </c>
+      <c r="D29" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E29" s="19" t="inlineStr">
         <is>
           <t>Submit/publish invoice</t>
         </is>
       </c>
-      <c r="F28" s="10" t="inlineStr">
+      <c r="F29" s="19" t="inlineStr">
         <is>
           <t>Invoice number is generated and invoice is due/visible to tenant</t>
         </is>
       </c>
-      <c r="G28" s="10" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H28" s="10" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I28" s="10" t="n"/>
-    </row>
-    <row r="29" ht="45" customHeight="1">
-      <c r="A29" s="10" t="inlineStr">
+      <c r="G29" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H29" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I29" s="19" t="n"/>
+    </row>
+    <row r="30" ht="45" customHeight="1">
+      <c r="A30" s="19" t="inlineStr">
         <is>
           <t>TC-04</t>
         </is>
       </c>
-      <c r="B29" s="10" t="inlineStr">
+      <c r="B30" s="19" t="inlineStr">
         <is>
           <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
         </is>
       </c>
-      <c r="C29" s="10" t="n">
-        <v>21</v>
-      </c>
-      <c r="D29" s="10" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E29" s="10" t="inlineStr">
+      <c r="C30" s="19" t="n">
+        <v>22</v>
+      </c>
+      <c r="D30" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E30" s="19" t="inlineStr">
         <is>
           <t>Logout</t>
         </is>
       </c>
-      <c r="F29" s="10" t="inlineStr">
+      <c r="F30" s="19" t="inlineStr">
         <is>
           <t>Login page is displayed</t>
         </is>
       </c>
-      <c r="G29" s="10" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H29" s="10" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I29" s="10" t="n"/>
-    </row>
-    <row r="30" ht="45" customHeight="1">
-      <c r="A30" s="10" t="inlineStr">
+      <c r="G30" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H30" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I30" s="19" t="n"/>
+    </row>
+    <row r="31" ht="45" customHeight="1">
+      <c r="A31" s="19" t="inlineStr">
         <is>
           <t>TC-04</t>
         </is>
       </c>
-      <c r="B30" s="10" t="inlineStr">
+      <c r="B31" s="19" t="inlineStr">
         <is>
           <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
         </is>
       </c>
-      <c r="C30" s="10" t="n">
-        <v>22</v>
-      </c>
-      <c r="D30" s="10" t="inlineStr">
+      <c r="C31" s="19" t="n">
+        <v>23</v>
+      </c>
+      <c r="D31" s="19" t="inlineStr">
         <is>
           <t>Tenant</t>
         </is>
       </c>
-      <c r="E30" s="10" t="inlineStr">
+      <c r="E31" s="19" t="inlineStr">
         <is>
           <t>Login, open tenant invoices, open created invoice, click Pay Online and Pay with Razorpay</t>
         </is>
       </c>
-      <c r="F30" s="10" t="inlineStr">
+      <c r="F31" s="19" t="inlineStr">
         <is>
           <t>Razorpay checkout opens</t>
         </is>
       </c>
-      <c r="G30" s="10" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H30" s="10" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I30" s="10" t="n"/>
-    </row>
-    <row r="31" ht="45" customHeight="1">
-      <c r="A31" s="10" t="inlineStr">
+      <c r="G31" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H31" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I31" s="19" t="n"/>
+    </row>
+    <row r="32" ht="45" customHeight="1">
+      <c r="A32" s="19" t="inlineStr">
         <is>
           <t>TC-04</t>
         </is>
       </c>
-      <c r="B31" s="10" t="inlineStr">
+      <c r="B32" s="19" t="inlineStr">
         <is>
           <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
         </is>
       </c>
-      <c r="C31" s="10" t="n">
-        <v>23</v>
-      </c>
-      <c r="D31" s="10" t="inlineStr">
+      <c r="C32" s="19" t="n">
+        <v>24</v>
+      </c>
+      <c r="D32" s="19" t="inlineStr">
         <is>
           <t>Tenant</t>
         </is>
       </c>
-      <c r="E31" s="10" t="inlineStr">
+      <c r="E32" s="19" t="inlineStr">
         <is>
           <t>Complete test payment using Netbanking -&gt; Bank of Baroda -&gt; Success</t>
         </is>
       </c>
-      <c r="F31" s="10" t="inlineStr">
+      <c r="F32" s="19" t="inlineStr">
         <is>
           <t>Invoice status becomes PAID</t>
         </is>
       </c>
-      <c r="G31" s="10" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H31" s="10" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I31" s="10" t="n"/>
-    </row>
-    <row r="32" ht="45" customHeight="1">
-      <c r="A32" s="10" t="inlineStr">
+      <c r="G32" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H32" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I32" s="19" t="n"/>
+    </row>
+    <row r="33" ht="45" customHeight="1">
+      <c r="A33" s="19" t="inlineStr">
         <is>
           <t>TC-04</t>
         </is>
       </c>
-      <c r="B32" s="10" t="inlineStr">
+      <c r="B33" s="19" t="inlineStr">
         <is>
           <t>Flow 1 with New Organization - tenant onboarding and rent collection</t>
         </is>
       </c>
-      <c r="C32" s="10" t="n">
-        <v>24</v>
-      </c>
-      <c r="D32" s="10" t="inlineStr">
+      <c r="C33" s="19" t="n">
+        <v>25</v>
+      </c>
+      <c r="D33" s="19" t="inlineStr">
         <is>
           <t>System</t>
         </is>
       </c>
-      <c r="E32" s="10" t="inlineStr">
+      <c r="E33" s="19" t="inlineStr">
         <is>
           <t>Save tenant details to test-data/tenant-new-org.json for Flow 2 New Org reuse</t>
         </is>
       </c>
-      <c r="F32" s="10" t="inlineStr">
+      <c r="F33" s="19" t="inlineStr">
         <is>
           <t>tenant-new-org.json is available for Flow2-NewOrganization</t>
         </is>
       </c>
-      <c r="G32" s="10" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H32" s="10" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I32" s="10" t="n"/>
+      <c r="G33" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H33" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I33" s="19" t="n"/>
     </row>
   </sheetData>
+  <autoFilter ref="A8:I33"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -5804,4 +5958,1329 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:I13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>Creating Contacts and Leads (4 each, separate random data)</t>
+        </is>
+      </c>
+      <c r="B1" s="16" t="n"/>
+      <c r="C1" s="16" t="n"/>
+      <c r="D1" s="16" t="n"/>
+      <c r="E1" s="16" t="n"/>
+      <c r="F1" s="16" t="n"/>
+      <c r="G1" s="16" t="n"/>
+      <c r="H1" s="16" t="n"/>
+      <c r="I1" s="16" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="16" t="n"/>
+      <c r="B2" s="16" t="n"/>
+      <c r="C2" s="16" t="n"/>
+      <c r="D2" s="16" t="n"/>
+      <c r="E2" s="16" t="n"/>
+      <c r="F2" s="16" t="n"/>
+      <c r="G2" s="16" t="n"/>
+      <c r="H2" s="16" t="n"/>
+      <c r="I2" s="16" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="17" t="inlineStr">
+        <is>
+          <t>Test ID</t>
+        </is>
+      </c>
+      <c r="B3" s="16" t="inlineStr">
+        <is>
+          <t>TC-06</t>
+        </is>
+      </c>
+      <c r="C3" s="16" t="n"/>
+      <c r="D3" s="16" t="n"/>
+      <c r="E3" s="16" t="n"/>
+      <c r="F3" s="16" t="n"/>
+      <c r="G3" s="16" t="n"/>
+      <c r="H3" s="16" t="n"/>
+      <c r="I3" s="16" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="n"/>
+      <c r="D4" s="16" t="n"/>
+      <c r="E4" s="16" t="n"/>
+      <c r="F4" s="16" t="n"/>
+      <c r="G4" s="16" t="n"/>
+      <c r="H4" s="16" t="n"/>
+      <c r="I4" s="16" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>End-to-end / Regression</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="n"/>
+      <c r="D5" s="16" t="n"/>
+      <c r="E5" s="16" t="n"/>
+      <c r="F5" s="16" t="n"/>
+      <c r="G5" s="16" t="n"/>
+      <c r="H5" s="16" t="n"/>
+      <c r="I5" s="16" t="n"/>
+    </row>
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>TC-03 completed successfully and test-data/org.json exists with valid Super Admin credentials.</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="n"/>
+      <c r="D6" s="16" t="n"/>
+      <c r="E6" s="16" t="n"/>
+      <c r="F6" s="16" t="n"/>
+      <c r="G6" s="16" t="n"/>
+      <c r="H6" s="16" t="n"/>
+      <c r="I6" s="16" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="16" t="n"/>
+      <c r="B7" s="16" t="n"/>
+      <c r="C7" s="16" t="n"/>
+      <c r="D7" s="16" t="n"/>
+      <c r="E7" s="16" t="n"/>
+      <c r="F7" s="16" t="n"/>
+      <c r="G7" s="16" t="n"/>
+      <c r="H7" s="16" t="n"/>
+      <c r="I7" s="16" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Test ID</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Step #</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>Actor</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="45" customHeight="1">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>TC-06</t>
+        </is>
+      </c>
+      <c r="B9" s="19" t="inlineStr">
+        <is>
+          <t>Creating Contacts and Leads (4 each, separate random data)</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E9" s="19" t="inlineStr">
+        <is>
+          <t>Login using orgId, email, and password from test-data/org.json</t>
+        </is>
+      </c>
+      <c r="F9" s="19" t="inlineStr">
+        <is>
+          <t>Admin session starts after leaving /login</t>
+        </is>
+      </c>
+      <c r="G9" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H9" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I9" s="19" t="inlineStr">
+        <is>
+          <t>TC-03 completed successfully and test-data/org.json exists with valid Super Admin credentials.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1">
+      <c r="A10" s="19" t="inlineStr">
+        <is>
+          <t>TC-06</t>
+        </is>
+      </c>
+      <c r="B10" s="19" t="inlineStr">
+        <is>
+          <t>Creating Contacts and Leads (4 each, separate random data)</t>
+        </is>
+      </c>
+      <c r="C10" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E10" s="19" t="inlineStr">
+        <is>
+          <t>Dismiss End-to-End Flow tour and Notifications modal if shown</t>
+        </is>
+      </c>
+      <c r="F10" s="19" t="inlineStr">
+        <is>
+          <t>UI is usable</t>
+        </is>
+      </c>
+      <c r="G10" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H10" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I10" s="19" t="n"/>
+    </row>
+    <row r="11" ht="45" customHeight="1">
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>TC-06</t>
+        </is>
+      </c>
+      <c r="B11" s="19" t="inlineStr">
+        <is>
+          <t>Creating Contacts and Leads (4 each, separate random data)</t>
+        </is>
+      </c>
+      <c r="C11" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="D11" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E11" s="19" t="inlineStr">
+        <is>
+          <t>Go to CRM -&gt; Contacts and create 4 contacts with unique random full name (contact*), email @yopmail.com, and mobile</t>
+        </is>
+      </c>
+      <c r="F11" s="19" t="inlineStr">
+        <is>
+          <t>Four contacts appear in Contacts Management</t>
+        </is>
+      </c>
+      <c r="G11" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H11" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I11" s="19" t="n"/>
+    </row>
+    <row r="12" ht="45" customHeight="1">
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>TC-06</t>
+        </is>
+      </c>
+      <c r="B12" s="19" t="inlineStr">
+        <is>
+          <t>Creating Contacts and Leads (4 each, separate random data)</t>
+        </is>
+      </c>
+      <c r="C12" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="D12" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E12" s="19" t="inlineStr">
+        <is>
+          <t>Go to CRM -&gt; Leads. For each of 4 different random leads (lead*), search the name, click Create New Lead, fill email/mobile, Create, then Convert to Deal with a random Payment Type</t>
+        </is>
+      </c>
+      <c r="F12" s="19" t="inlineStr">
+        <is>
+          <t>Four leads are converted to deals</t>
+        </is>
+      </c>
+      <c r="G12" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H12" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I12" s="19" t="n"/>
+    </row>
+    <row r="13" ht="45" customHeight="1">
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t>TC-06</t>
+        </is>
+      </c>
+      <c r="B13" s="19" t="inlineStr">
+        <is>
+          <t>Creating Contacts and Leads (4 each, separate random data)</t>
+        </is>
+      </c>
+      <c r="C13" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="D13" s="19" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="E13" s="19" t="inlineStr">
+        <is>
+          <t>Save contacts and leads to test-data/crm-contacts-leads.json</t>
+        </is>
+      </c>
+      <c r="F13" s="19" t="inlineStr">
+        <is>
+          <t>crm-contacts-leads.json is available for ExistingContact-ToTenantPayment (TC-07)</t>
+        </is>
+      </c>
+      <c r="G13" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H13" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I13" s="19" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A8:I13"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:I26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="B1" s="16" t="n"/>
+      <c r="C1" s="16" t="n"/>
+      <c r="D1" s="16" t="n"/>
+      <c r="E1" s="16" t="n"/>
+      <c r="F1" s="16" t="n"/>
+      <c r="G1" s="16" t="n"/>
+      <c r="H1" s="16" t="n"/>
+      <c r="I1" s="16" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="16" t="n"/>
+      <c r="B2" s="16" t="n"/>
+      <c r="C2" s="16" t="n"/>
+      <c r="D2" s="16" t="n"/>
+      <c r="E2" s="16" t="n"/>
+      <c r="F2" s="16" t="n"/>
+      <c r="G2" s="16" t="n"/>
+      <c r="H2" s="16" t="n"/>
+      <c r="I2" s="16" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="17" t="inlineStr">
+        <is>
+          <t>Test ID</t>
+        </is>
+      </c>
+      <c r="B3" s="16" t="inlineStr">
+        <is>
+          <t>TC-07</t>
+        </is>
+      </c>
+      <c r="C3" s="16" t="n"/>
+      <c r="D3" s="16" t="n"/>
+      <c r="E3" s="16" t="n"/>
+      <c r="F3" s="16" t="n"/>
+      <c r="G3" s="16" t="n"/>
+      <c r="H3" s="16" t="n"/>
+      <c r="I3" s="16" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="n"/>
+      <c r="D4" s="16" t="n"/>
+      <c r="E4" s="16" t="n"/>
+      <c r="F4" s="16" t="n"/>
+      <c r="G4" s="16" t="n"/>
+      <c r="H4" s="16" t="n"/>
+      <c r="I4" s="16" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>End-to-end / Regression</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="n"/>
+      <c r="D5" s="16" t="n"/>
+      <c r="E5" s="16" t="n"/>
+      <c r="F5" s="16" t="n"/>
+      <c r="G5" s="16" t="n"/>
+      <c r="H5" s="16" t="n"/>
+      <c r="I5" s="16" t="n"/>
+    </row>
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>TC-03 and TC-06 completed; test-data/org.json and test-data/crm-contacts-leads.json exist. Deal Approve workflow should already exist from TC-04 (Flow1-NewOrganization).</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="n"/>
+      <c r="D6" s="16" t="n"/>
+      <c r="E6" s="16" t="n"/>
+      <c r="F6" s="16" t="n"/>
+      <c r="G6" s="16" t="n"/>
+      <c r="H6" s="16" t="n"/>
+      <c r="I6" s="16" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="16" t="n"/>
+      <c r="B7" s="16" t="n"/>
+      <c r="C7" s="16" t="n"/>
+      <c r="D7" s="16" t="n"/>
+      <c r="E7" s="16" t="n"/>
+      <c r="F7" s="16" t="n"/>
+      <c r="G7" s="16" t="n"/>
+      <c r="H7" s="16" t="n"/>
+      <c r="I7" s="16" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Test ID</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Step #</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>Actor</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="45" customHeight="1">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>TC-07</t>
+        </is>
+      </c>
+      <c r="B9" s="19" t="inlineStr">
+        <is>
+          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E9" s="19" t="inlineStr">
+        <is>
+          <t>Login using orgId, email, and password from test-data/org.json</t>
+        </is>
+      </c>
+      <c r="F9" s="19" t="inlineStr">
+        <is>
+          <t>Admin session starts after leaving /login</t>
+        </is>
+      </c>
+      <c r="G9" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H9" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I9" s="19" t="inlineStr">
+        <is>
+          <t>TC-03 and TC-06 completed; test-data/org.json and test-data/crm-contacts-leads.json exist. Deal Approve workflow should already exist from TC-04 (Flow1-NewOrganization).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1">
+      <c r="A10" s="19" t="inlineStr">
+        <is>
+          <t>TC-07</t>
+        </is>
+      </c>
+      <c r="B10" s="19" t="inlineStr">
+        <is>
+          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C10" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E10" s="19" t="inlineStr">
+        <is>
+          <t>Open Accounts -&gt; Taxes. Delete VAT if present. Skip create if GST (18%) already exists; otherwise create GST (18%) / GST-18 / 18%</t>
+        </is>
+      </c>
+      <c r="F10" s="19" t="inlineStr">
+        <is>
+          <t>GST (18%) is available in tax dropdowns</t>
+        </is>
+      </c>
+      <c r="G10" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H10" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I10" s="19" t="n"/>
+    </row>
+    <row r="11" ht="45" customHeight="1">
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>TC-07</t>
+        </is>
+      </c>
+      <c r="B11" s="19" t="inlineStr">
+        <is>
+          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C11" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="D11" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E11" s="19" t="inlineStr">
+        <is>
+          <t>Go to CRM Contacts and open a random contact from crm-contacts-leads.json</t>
+        </is>
+      </c>
+      <c r="F11" s="19" t="inlineStr">
+        <is>
+          <t>Contact details page opens</t>
+        </is>
+      </c>
+      <c r="G11" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H11" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I11" s="19" t="n"/>
+    </row>
+    <row r="12" ht="45" customHeight="1">
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>TC-07</t>
+        </is>
+      </c>
+      <c r="B12" s="19" t="inlineStr">
+        <is>
+          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C12" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="D12" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E12" s="19" t="inlineStr">
+        <is>
+          <t>Click Create Lead (if lead already exists for this contact, open the existing lead or deal instead)</t>
+        </is>
+      </c>
+      <c r="F12" s="19" t="inlineStr">
+        <is>
+          <t>Lead details or Deal Details page is shown</t>
+        </is>
+      </c>
+      <c r="G12" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H12" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I12" s="19" t="n"/>
+    </row>
+    <row r="13" ht="45" customHeight="1">
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t>TC-07</t>
+        </is>
+      </c>
+      <c r="B13" s="19" t="inlineStr">
+        <is>
+          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C13" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="D13" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E13" s="19" t="inlineStr">
+        <is>
+          <t>If not already a deal, Convert to Deal and select a payment type</t>
+        </is>
+      </c>
+      <c r="F13" s="19" t="inlineStr">
+        <is>
+          <t>Deal Details page opens</t>
+        </is>
+      </c>
+      <c r="G13" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H13" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I13" s="19" t="n"/>
+    </row>
+    <row r="14" ht="45" customHeight="1">
+      <c r="A14" s="19" t="inlineStr">
+        <is>
+          <t>TC-07</t>
+        </is>
+      </c>
+      <c r="B14" s="19" t="inlineStr">
+        <is>
+          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C14" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="D14" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E14" s="19" t="inlineStr">
+        <is>
+          <t>If Add Property is enabled, click Add Property. In the dialog set Status combobox to Vacant, select one random vacant property, click Add Property. If Add Property is disabled, keep the property already on the deal</t>
+        </is>
+      </c>
+      <c r="F14" s="19" t="inlineStr">
+        <is>
+          <t>A vacant (or existing) property is on the deal</t>
+        </is>
+      </c>
+      <c r="G14" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H14" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I14" s="19" t="n"/>
+    </row>
+    <row r="15" ht="45" customHeight="1">
+      <c r="A15" s="19" t="inlineStr">
+        <is>
+          <t>TC-07</t>
+        </is>
+      </c>
+      <c r="B15" s="19" t="inlineStr">
+        <is>
+          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C15" s="19" t="n">
+        <v>7</v>
+      </c>
+      <c r="D15" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E15" s="19" t="inlineStr">
+        <is>
+          <t>On the deal property card set Property Rent (120000-600000 if 0), Discount % (10-30), Tax GST (18%), Save, mark Site visit done</t>
+        </is>
+      </c>
+      <c r="F15" s="19" t="inlineStr">
+        <is>
+          <t>Pricing is saved and site visit is done</t>
+        </is>
+      </c>
+      <c r="G15" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H15" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I15" s="19" t="n"/>
+    </row>
+    <row r="16" ht="45" customHeight="1">
+      <c r="A16" s="19" t="inlineStr">
+        <is>
+          <t>TC-07</t>
+        </is>
+      </c>
+      <c r="B16" s="19" t="inlineStr">
+        <is>
+          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C16" s="19" t="n">
+        <v>8</v>
+      </c>
+      <c r="D16" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E16" s="19" t="inlineStr">
+        <is>
+          <t>Click Submit for Approval (confirm dialog if shown), then Approve on Internal Approval and Confirm</t>
+        </is>
+      </c>
+      <c r="F16" s="19" t="inlineStr">
+        <is>
+          <t>Deal approval workflow completes</t>
+        </is>
+      </c>
+      <c r="G16" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H16" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I16" s="19" t="n"/>
+    </row>
+    <row r="17" ht="45" customHeight="1">
+      <c r="A17" s="19" t="inlineStr">
+        <is>
+          <t>TC-07</t>
+        </is>
+      </c>
+      <c r="B17" s="19" t="inlineStr">
+        <is>
+          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C17" s="19" t="n">
+        <v>9</v>
+      </c>
+      <c r="D17" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E17" s="19" t="inlineStr">
+        <is>
+          <t>Create/view contract and approve the contract</t>
+        </is>
+      </c>
+      <c r="F17" s="19" t="inlineStr">
+        <is>
+          <t>Contract is approved</t>
+        </is>
+      </c>
+      <c r="G17" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H17" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I17" s="19" t="n"/>
+    </row>
+    <row r="18" ht="45" customHeight="1">
+      <c r="A18" s="19" t="inlineStr">
+        <is>
+          <t>TC-07</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="inlineStr">
+        <is>
+          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C18" s="19" t="n">
+        <v>10</v>
+      </c>
+      <c r="D18" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E18" s="19" t="inlineStr">
+        <is>
+          <t>Create tenant user from Action Buttons tab</t>
+        </is>
+      </c>
+      <c r="F18" s="19" t="inlineStr">
+        <is>
+          <t>Tenant user is created; password captured from dialog or YOPmail</t>
+        </is>
+      </c>
+      <c r="G18" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H18" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I18" s="19" t="n"/>
+    </row>
+    <row r="19" ht="45" customHeight="1">
+      <c r="A19" s="19" t="inlineStr">
+        <is>
+          <t>TC-07</t>
+        </is>
+      </c>
+      <c r="B19" s="19" t="inlineStr">
+        <is>
+          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C19" s="19" t="n">
+        <v>11</v>
+      </c>
+      <c r="D19" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E19" s="19" t="inlineStr">
+        <is>
+          <t>Create move-in request with current move-in date; complete it in Operations Requests</t>
+        </is>
+      </c>
+      <c r="F19" s="19" t="inlineStr">
+        <is>
+          <t>Move-in request becomes completed</t>
+        </is>
+      </c>
+      <c r="G19" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H19" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I19" s="19" t="n"/>
+    </row>
+    <row r="20" ht="45" customHeight="1">
+      <c r="A20" s="19" t="inlineStr">
+        <is>
+          <t>TC-07</t>
+        </is>
+      </c>
+      <c r="B20" s="19" t="inlineStr">
+        <is>
+          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C20" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="D20" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E20" s="19" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+      <c r="F20" s="19" t="inlineStr">
+        <is>
+          <t>Login page is displayed</t>
+        </is>
+      </c>
+      <c r="G20" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H20" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I20" s="19" t="n"/>
+    </row>
+    <row r="21" ht="45" customHeight="1">
+      <c r="A21" s="19" t="inlineStr">
+        <is>
+          <t>TC-07</t>
+        </is>
+      </c>
+      <c r="B21" s="19" t="inlineStr">
+        <is>
+          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C21" s="19" t="n">
+        <v>13</v>
+      </c>
+      <c r="D21" s="19" t="inlineStr">
+        <is>
+          <t>Tenant</t>
+        </is>
+      </c>
+      <c r="E21" s="19" t="inlineStr">
+        <is>
+          <t>Login with generated tenant credentials (orgId from org.json)</t>
+        </is>
+      </c>
+      <c r="F21" s="19" t="inlineStr">
+        <is>
+          <t>Tenant portal opens successfully</t>
+        </is>
+      </c>
+      <c r="G21" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H21" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I21" s="19" t="n"/>
+    </row>
+    <row r="22" ht="45" customHeight="1">
+      <c r="A22" s="19" t="inlineStr">
+        <is>
+          <t>TC-07</t>
+        </is>
+      </c>
+      <c r="B22" s="19" t="inlineStr">
+        <is>
+          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C22" s="19" t="n">
+        <v>14</v>
+      </c>
+      <c r="D22" s="19" t="inlineStr">
+        <is>
+          <t>Tenant</t>
+        </is>
+      </c>
+      <c r="E22" s="19" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+      <c r="F22" s="19" t="inlineStr">
+        <is>
+          <t>Login page is displayed</t>
+        </is>
+      </c>
+      <c r="G22" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H22" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I22" s="19" t="n"/>
+    </row>
+    <row r="23" ht="45" customHeight="1">
+      <c r="A23" s="19" t="inlineStr">
+        <is>
+          <t>TC-07</t>
+        </is>
+      </c>
+      <c r="B23" s="19" t="inlineStr">
+        <is>
+          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C23" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="D23" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E23" s="19" t="inlineStr">
+        <is>
+          <t>Login again and create rent invoice: item rent, Chart of Account 4000 - Rental Income, amount from deal rent; submit/publish</t>
+        </is>
+      </c>
+      <c r="F23" s="19" t="inlineStr">
+        <is>
+          <t>Invoice is due/visible to tenant</t>
+        </is>
+      </c>
+      <c r="G23" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H23" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I23" s="19" t="n"/>
+    </row>
+    <row r="24" ht="45" customHeight="1">
+      <c r="A24" s="19" t="inlineStr">
+        <is>
+          <t>TC-07</t>
+        </is>
+      </c>
+      <c r="B24" s="19" t="inlineStr">
+        <is>
+          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C24" s="19" t="n">
+        <v>16</v>
+      </c>
+      <c r="D24" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E24" s="19" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+      <c r="F24" s="19" t="inlineStr">
+        <is>
+          <t>Login page is displayed</t>
+        </is>
+      </c>
+      <c r="G24" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H24" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I24" s="19" t="n"/>
+    </row>
+    <row r="25" ht="45" customHeight="1">
+      <c r="A25" s="19" t="inlineStr">
+        <is>
+          <t>TC-07</t>
+        </is>
+      </c>
+      <c r="B25" s="19" t="inlineStr">
+        <is>
+          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C25" s="19" t="n">
+        <v>17</v>
+      </c>
+      <c r="D25" s="19" t="inlineStr">
+        <is>
+          <t>Tenant</t>
+        </is>
+      </c>
+      <c r="E25" s="19" t="inlineStr">
+        <is>
+          <t>Login, open the invoice, Pay Online / Pay with Razorpay, Netbanking -&gt; Bank of Baroda -&gt; Success</t>
+        </is>
+      </c>
+      <c r="F25" s="19" t="inlineStr">
+        <is>
+          <t>Invoice status becomes PAID</t>
+        </is>
+      </c>
+      <c r="G25" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H25" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I25" s="19" t="n"/>
+    </row>
+    <row r="26" ht="45" customHeight="1">
+      <c r="A26" s="19" t="inlineStr">
+        <is>
+          <t>TC-07</t>
+        </is>
+      </c>
+      <c r="B26" s="19" t="inlineStr">
+        <is>
+          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C26" s="19" t="n">
+        <v>18</v>
+      </c>
+      <c r="D26" s="19" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="E26" s="19" t="inlineStr">
+        <is>
+          <t>Save tenant details to test-data/tenant-new-org.json</t>
+        </is>
+      </c>
+      <c r="F26" s="19" t="inlineStr">
+        <is>
+          <t>tenant-new-org.json is updated for optional Flow 2 reuse</t>
+        </is>
+      </c>
+      <c r="G26" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H26" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I26" s="19" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A8:I26"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add full chain test script and new test for Direct Lead to Tenant Payment
- Introduced a new script to run all PropExcel specs sequentially, ensuring isolated output for each test.
- Added a comprehensive test for the Direct Lead to Tenant Payment flow, including detailed data generation and payment handling via Razorpay.
- Updated package.json to include the new test script for easier execution.
</commit_message>
<xml_diff>
--- a/PropExcel_Test_Cases.xlsx
+++ b/PropExcel_Test_Cases.xlsx
@@ -8,18 +8,21 @@
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="TC-01_Flow1" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="TC-02_Flow2" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="TC-03_CreateOrganization" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="TC-04_Flow1_NewOrg" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="TC-05_Flow2_NewOrg" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="TC-06_ContactsLeadsDeals" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="TC-07_ExistingContactPayment" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="TC-00_Cleanup" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="TC-01_Flow1" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="TC-02_Flow2" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="TC-03_CreateOrganization" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="TC-04_Flow1_NewOrg" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="TC-05_Flow2_NewOrg" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="TC-06_ContactsLeadsDeals" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="TC-07_ExistingContactPayment" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="TC-08_SkipLeadPayment" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="TC-09_DirectLeadPayment" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'TC-04_Flow1_NewOrg'!$A$8:$I$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'TC-06_ContactsLeadsDeals'!$A$8:$I$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'TC-07_ExistingContactPayment'!$A$8:$I$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'TC-04_Flow1_NewOrg'!$A$8:$I$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'TC-06_ContactsLeadsDeals'!$A$8:$I$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'TC-07_ExistingContactPayment'!$A$8:$I$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -531,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -545,6 +548,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -577,7 +581,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Legacy: test240 | New Org: dynamic org from test-data/org.json</t>
+          <t>Existing org: test (test@yopmail.com / Test2026$) | New Org: dynamic org from test-data/org.json</t>
         </is>
       </c>
     </row>
@@ -601,7 +605,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>tests/Flow1-ExistingOrganization.spec.ts, tests/Flow2-ExistingOrganization.spec.ts, tests/CreateOrganization.spec.ts, tests/Flow1-NewOrganization.spec.ts, tests/Creating Contacts,Leads,Deals.spec.ts, tests/ExistingContact-ToTenantPayment.spec.ts, tests/Flow2-NewOrganization.spec.ts</t>
+          <t>tests/Cleanup Scenario.spec.ts, tests/CreateOrganization.spec.ts, tests/Flow1-ExistingOrganization.spec.ts, tests/Flow2-ExistingOrganization.spec.ts, tests/Flow1-NewOrganization.spec.ts, tests/Flow2-NewOrganization.spec.ts, tests/Creating Contacts,Leads,Deals.spec.ts, tests/ExistingContact-ToTenantPayment.spec.ts, tests/Skip lead flow - tenenat Payment.spec.ts, tests/Direct Lead to Tenant Payment.spec.ts</t>
         </is>
       </c>
     </row>
@@ -613,7 +617,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Legacy: Flow 1 (Flow1-ExistingOrganization) -&gt; Flow 2 (Flow2-ExistingOrganization). New Org chain: Create Organization -&gt; Flow1-NewOrganization -&gt; Creating Contacts,Leads,Deals -&gt; ExistingContact-ToTenantPayment. Optional: Flow2-NewOrganization after Flow1 (uses tenant-new-org.json).</t>
+          <t>New Org chain: TC-00 Cleanup -&gt; TC-03 CreateOrganization -&gt; TC-04 Flow1-NewOrganization -&gt; TC-06 Creating Contacts,Leads,Deals -&gt; TC-07 ExistingContact-ToTenantPayment -&gt; TC-08 Skip lead flow -&gt; TC-09 Direct Lead to Tenant Payment -&gt; TC-05 Flow2-NewOrganization (optional). Existing org chain: TC-01 Flow1-ExistingOrganization -&gt; TC-02 Flow2-ExistingOrganization.</t>
         </is>
       </c>
     </row>
@@ -625,10 +629,12 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Automated organization registration, CRM contacts/leads/deals, tenant onboarding, rent collection, service request, vendor billing, tenant invoicing, and Razorpay payment journeys for both existing (test240) and newly created organizations</t>
-        </is>
-      </c>
-    </row>
+          <t>Automated platform cleanup, organization registration, CRM contacts/leads/deals, tenant onboarding, rent collection, service request, vendor billing, tenant invoicing, and Razorpay payment journeys for both existing org (test) and newly created organizations. Tenant credentials via IMAP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10"/>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
@@ -640,87 +646,130 @@
     <row r="13" ht="32" customHeight="1">
       <c r="A13" s="11" t="inlineStr">
         <is>
-          <t>TC-01</t>
+          <t>TC-00</t>
         </is>
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>Create property, onboard tenant, create rent invoice, tenant pays via Razorpay (org: test240). Script: Flow1-ExistingOrganization.spec.ts</t>
+          <t>Delete auto organizations (platform admin). Script: Cleanup Scenario.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1">
       <c r="A14" s="11" t="inlineStr">
         <is>
-          <t>TC-02</t>
+          <t>TC-01</t>
         </is>
       </c>
       <c r="B14" s="12" t="inlineStr">
         <is>
-          <t>Tenant request -&gt; vendor -&gt; task -&gt; tenant approval -&gt; vendor bill paid -&gt; tenant service invoice paid (org: test240). Script: Flow2-ExistingOrganization.spec.ts</t>
+          <t>Create property, onboard tenant, rent invoice, Razorpay pay (org: test). Script: Flow1-ExistingOrganization.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="15" ht="32" customHeight="1">
       <c r="A15" s="13" t="inlineStr">
         <is>
-          <t>TC-03</t>
+          <t>TC-02</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>Create new organization via registration + Stripe card verification; save credentials to org.json. Script: CreateOrganization.spec.ts</t>
+          <t>Tenant request -&gt; vendor -&gt; task -&gt; approval -&gt; bill -&gt; invoice -&gt; Razorpay (org: test). Script: Flow2-ExistingOrganization.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="16" ht="32" customHeight="1">
       <c r="A16" s="13" t="inlineStr">
         <is>
-          <t>TC-04</t>
+          <t>TC-03</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>New-org Flow 1: Razorpay, GST 18% tax, Deal Approve workflow, create property, onboard tenant, rent invoice, Razorpay pay; save tenant-new-org.json. Script: Flow1-NewOrganization.spec.ts</t>
+          <t>Create new organization via Stripe; save org.json. Script: CreateOrganization.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="17" ht="32" customHeight="1">
       <c r="A17" s="13" t="inlineStr">
         <is>
-          <t>TC-05</t>
+          <t>TC-04</t>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
         <is>
-          <t>New-org Flow 2: tenant request -&gt; vendor -&gt; task -&gt; approval -&gt; bill paid -&gt; service invoice paid (uses org.json + tenant-new-org.json). Script: Flow2-NewOrganization.spec.ts</t>
+          <t>New-org Flow 1: Razorpay, GST, Deal Approve, property, tenant, invoice, Razorpay. Script: Flow1-NewOrganization.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="18" ht="32" customHeight="1">
       <c r="A18" s="13" t="inlineStr">
         <is>
-          <t>TC-06</t>
+          <t>TC-05</t>
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
         <is>
-          <t>Create 4 contacts and 4 leads (separate random data); convert each lead to a deal; save crm-contacts-leads.json. Script: Creating Contacts,Leads,Deals.spec.ts</t>
+          <t>New-org Flow 2: request, vendor, task, bill, invoice, Razorpay. Script: Flow2-NewOrganization.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="19" ht="32" customHeight="1">
       <c r="A19" s="13" t="inlineStr">
         <is>
+          <t>TC-06</t>
+        </is>
+      </c>
+      <c r="B19" s="14" t="inlineStr">
+        <is>
+          <t>Create 4 contacts + 4 leads (tenantN sequential); save crm-contacts-leads.json. Script: Creating Contacts,Leads,Deals.spec.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>TC-07</t>
         </is>
       </c>
-      <c r="B19" s="14" t="inlineStr">
-        <is>
-          <t>Existing CRM contact -&gt; lead/deal -&gt; Vacant property -&gt; GST 18% pricing -&gt; approval workflow -&gt; tenant -&gt; rent invoice paid. Script: ExistingContact-ToTenantPayment.spec.ts</t>
-        </is>
-      </c>
-    </row>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Existing CRM contact -&gt; lead/deal -&gt; tenant -&gt; rent invoice paid. Script: ExistingContact-ToTenantPayment.spec.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>TC-08</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Skip lead: existing contact -&gt; Create Deal -&gt; tenant -&gt; rent payment. Script: Skip lead flow - tenenat Payment.spec.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>TC-09</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Direct lead: auto contact -&gt; deal -&gt; tenant -&gt; rent payment. Script: Direct Lead to Tenant Payment.spec.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:B1"/>
@@ -729,7 +778,1707 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Skip lead - existing contact Create Deal through rent payment (new org)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Test ID</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>TC-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>End-to-end / Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>TC-03 and TC-06 completed; org.json and crm-contacts-leads.json exist.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Script</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>tests/Skip lead flow - tenenat Payment.spec.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Test ID</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Step #</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Actor</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TC-08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Skip lead - existing contact Create Deal through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Login using orgId, email, password from test-data/org.json</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Admin session starts</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>TC-03 and TC-06 completed; org.json and crm-contacts-leads.json exist.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>TC-08</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Skip lead - existing contact Create Deal through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Configure Razorpay integration and tax settings (GST 18%) if not already done</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Payment and tax setup complete</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TC-08</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Skip lead - existing contact Create Deal through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>3</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>CRM -&gt; Deals -&gt; Create Deal with shared contact from crm-contacts-leads.json (skip lead creation)</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Deal form opens with contact selected</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>TC-08</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Skip lead - existing contact Create Deal through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>4</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Add vacant property to deal, set rent/discount/GST, mark site visit done</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Deal property pricing saved</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>TC-08</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Skip lead - existing contact Create Deal through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>5</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Submit for Approval and complete Deal Approve workflow</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Deal is approved</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>TC-08</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Skip lead - existing contact Create Deal through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>6</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Create/view contract and approve contract</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Contract approved</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>TC-08</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Skip lead - existing contact Create Deal through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>7</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Create tenant user; password from dialog or IMAP</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Tenant user created</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>TC-08</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Skip lead - existing contact Create Deal through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>8</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Create move-in request and complete in Operations Requests</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Move-in completed</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>TC-08</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Skip lead - existing contact Create Deal through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>9</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Login page displayed</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>TC-08</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Skip lead - existing contact Create Deal through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Tenant</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Login with tenant credentials (IMAP or captured password)</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Tenant portal opens</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>TC-08</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Skip lead - existing contact Create Deal through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>11</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Tenant</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Login page displayed</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>TC-08</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Skip lead - existing contact Create Deal through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>12</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Create rent invoice (4000 Rental Income), submit/publish</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Invoice visible to tenant</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>TC-08</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Skip lead - existing contact Create Deal through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>13</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Login page displayed</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>TC-08</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Skip lead - existing contact Create Deal through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>14</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Tenant</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Pay invoice via Razorpay Netbanking -&gt; Bank of Baroda -&gt; Success</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Invoice status PAID</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Direct Lead - auto contact through rent payment (new org)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Test ID</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>TC-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>End-to-end / Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>TC-03 completed; org.json exists with valid Super Admin credentials.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Script</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>tests/Direct Lead to Tenant Payment.spec.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Test ID</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Step #</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Actor</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TC-09</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Direct Lead - auto contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Login using orgId, email, password from test-data/org.json</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Admin session starts</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>TC-03 completed; org.json exists with valid Super Admin credentials.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>TC-09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Direct Lead - auto contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>CRM -&gt; Leads -&gt; Create New Lead: search tenantN name, No matches -&gt; Create New Lead</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Lead create form opens</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TC-09</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Direct Lead - auto contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>3</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Fill lead form (name, email propexceltest+tenantN@gmail.com, India mobile, nationality), Create</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Lead details page opens (contact auto-created)</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>TC-09</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Direct Lead - auto contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>4</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Convert to Deal, select payment type</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Deal Details page opens</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>TC-09</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Direct Lead - auto contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>5</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Add property to deal, set tax, Approve deal</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Deal approved</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>TC-09</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Direct Lead - auto contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>6</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Create/view contract and approve contract</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Contract approved</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>TC-09</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Direct Lead - auto contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>7</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Create tenant user; password from dialog or IMAP</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Tenant user created</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>TC-09</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Direct Lead - auto contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>8</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Create move-in request and complete in Operations</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Move-in completed</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>TC-09</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Direct Lead - auto contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>9</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Login page displayed</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>TC-09</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Direct Lead - auto contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Tenant</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Login with tenant credentials (IMAP or captured password)</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Tenant portal opens</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>TC-09</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Direct Lead - auto contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>11</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Tenant</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Login page displayed</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>TC-09</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Direct Lead - auto contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>12</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Create rent invoice (4000 Rental Income), submit/publish</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Invoice visible to tenant</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>TC-09</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Direct Lead - auto contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>13</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Login page displayed</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>TC-09</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Direct Lead - auto contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>14</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Tenant</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Pay invoice via Razorpay Netbanking -&gt; Bank of Baroda -&gt; Success</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Invoice status PAID</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Cleanup Scenario - delete auto organizations</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Test ID</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>TC-00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>End-to-end / Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Platform admin credentials valid: propexcel / admin@propexcel.com / Demo2026$</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Script</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>tests/Cleanup Scenario.spec.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Test ID</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Step #</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Actor</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TC-00</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Cleanup Scenario - delete auto organizations</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Platform Admin</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Login at https://test.propexcel.com/login with org propexcel, admin@propexcel.com, Demo2026$</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Admin session starts</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Platform admin credentials valid: propexcel / admin@propexcel.com / Demo2026$</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>TC-00</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Cleanup Scenario - delete auto organizations</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Platform Admin</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Navigate to Organizations list (search organizations)</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Organizations page is displayed</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TC-00</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Cleanup Scenario - delete auto organizations</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>3</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Platform Admin</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Search organizations matching "Auto" and delete each (confirm dialog)</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>All matching auto orgs are deleted</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>TC-00</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Cleanup Scenario - delete auto organizations</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>4</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Platform Admin</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Login page is displayed</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -756,6 +2505,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -800,10 +2550,11 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Super Admin credentials are valid and TEST environment is available.</t>
-        </is>
-      </c>
-    </row>
+          <t>Existing org Super Admin credentials valid: org test, email test@yopmail.com, password Test2026$. TEST environment available. GMAIL_APP_PASSWORD set for IMAP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
@@ -872,7 +2623,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Login with org test240 using admin credentials</t>
+          <t>Login with org test, email test@yopmail.com, password Test2026$</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -892,7 +2643,7 @@
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Super Admin credentials are valid and TEST environment is available.</t>
+          <t>Existing org Super Admin credentials valid: org test, email test@yopmail.com, password Test2026$. TEST environment available. GMAIL_APP_PASSWORD set for IMAP.</t>
         </is>
       </c>
     </row>
@@ -958,7 +2709,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Go to CRM Contacts and create a new contact with generated tenant details</t>
+          <t>Go to CRM Contacts and create contact (or reuse if duplicate) with tenantN name, propexceltest+tenantN@gmail.com, India mobile, Indian nationality</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -999,7 +2750,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Open contact and create lead</t>
+          <t>Open contact and create lead (or open existing lead if duplicate email/phone exists)</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -1209,7 +2960,7 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Tenant user is created and password is captured from dialog or YOPmail</t>
+          <t>Tenant user is created and password is captured from dialog or IMAP (Gmail app password)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1368,7 +3119,7 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Login with generated tenant credentials from YOPmail or captured password</t>
+          <t>Login with generated tenant credentials from IMAP (Gmail app password) or captured password</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
@@ -1724,7 +3475,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1751,6 +3502,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -1795,10 +3547,11 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>TC-01 completed successfully and test-data/tenant.json exists with valid tenant credentials.</t>
-        </is>
-      </c>
-    </row>
+          <t>TC-01 completed; test-data/tenant.json exists with orgId test and valid tenant credentials.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
@@ -1887,7 +3640,7 @@
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>TC-01 completed successfully and test-data/tenant.json exists with valid tenant credentials.</t>
+          <t>TC-01 completed; test-data/tenant.json exists with orgId test and valid tenant credentials.</t>
         </is>
       </c>
     </row>
@@ -1994,7 +3747,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Login using admin credentials</t>
+          <t>Login as Super Admin: org test, email test@yopmail.com, password Test2026$</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -2199,7 +3952,7 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Add task with task title, status Open, random priority, and assign the created vendor</t>
+          <t>Add task with status Open, random priority, assign created vendor (fallback: Super Admin if vendor not in dropdown yet)</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -2924,7 +4677,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2951,6 +4704,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
@@ -2999,6 +4753,7 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
@@ -3153,7 +4908,7 @@
       </c>
       <c r="E11" s="10" t="inlineStr">
         <is>
-          <t>Enter Organization Name as Automation ###, Organization Code as automation-###, admin email as automation###@yopmail.com, password Test2026$, and referral code TEST9</t>
+          <t>Enter Organization Name as Automation ###, Organization Code as automation-###, admin email as automation###@gmail.com (propexceltest+tenantN).com, password Test2026$, and referral code TEST9</t>
         </is>
       </c>
       <c r="F11" s="10" t="inlineStr">
@@ -3547,7 +5302,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4249,7 +6004,7 @@
       </c>
       <c r="F21" s="19" t="inlineStr">
         <is>
-          <t>Tenant user is created and password is captured from dialog or YOPmail</t>
+          <t>Tenant user is created and password is captured from dialog or IMAP (Gmail app password)</t>
         </is>
       </c>
       <c r="G21" s="19" t="inlineStr">
@@ -4408,7 +6163,7 @@
       </c>
       <c r="E25" s="19" t="inlineStr">
         <is>
-          <t>Login with generated tenant credentials (orgId from org.json) from YOPmail or captured password</t>
+          <t>Login with generated tenant credentials (orgId from org.json) from IMAP (Gmail app password) or captured password</t>
         </is>
       </c>
       <c r="F25" s="19" t="inlineStr">
@@ -4763,7 +6518,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4790,6 +6545,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
@@ -4838,6 +6594,7 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
@@ -5960,7 +7717,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6247,7 +8004,7 @@
       </c>
       <c r="E11" s="19" t="inlineStr">
         <is>
-          <t>Go to CRM -&gt; Contacts and create 4 contacts with unique random full name (contact*), email @yopmail.com, and mobile</t>
+          <t>Go to CRM -&gt; Contacts and create 4 contacts (tenantN sequential): fullName tenantN, email propexceltest+tenantN@gmail.com, India mobile, Indian nationality</t>
         </is>
       </c>
       <c r="F11" s="19" t="inlineStr">
@@ -6356,7 +8113,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6935,7 +8692,7 @@
       </c>
       <c r="F18" s="19" t="inlineStr">
         <is>
-          <t>Tenant user is created; password captured from dialog or YOPmail</t>
+          <t>Tenant user is created; password captured from dialog or IMAP (Gmail app password)</t>
         </is>
       </c>
       <c r="G18" s="19" t="inlineStr">
@@ -7053,7 +8810,7 @@
       </c>
       <c r="E21" s="19" t="inlineStr">
         <is>
-          <t>Login with generated tenant credentials (orgId from org.json)</t>
+          <t>Login with tenant credentials from IMAP or captured password (orgId from org.json)</t>
         </is>
       </c>
       <c r="F21" s="19" t="inlineStr">

</xml_diff>

<commit_message>
- Increased timeout settings for tests to improve stability and performance. - Updated screenshot and video capture settings to optimize test execution. - Refactored test scripts to streamline the execution of the full regression chain, adding a new script for resuming tests from a specific step. - Introduced new test cases for existing contact and deal workflows, ensuring comprehensive coverage of payment processes. - Updated test case descriptions and improved data handling in the Excel test cases file.
</commit_message>
<xml_diff>
--- a/PropExcel_Test_Cases.xlsx
+++ b/PropExcel_Test_Cases.xlsx
@@ -15,14 +15,15 @@
     <sheet name="TC-04_Flow1_NewOrg" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="TC-05_Flow2_NewOrg" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="TC-06_ContactsLeadsDeals" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="TC-07_ExistingContactPayment" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="TC-08_SkipLeadPayment" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="TC-09_DirectLeadPayment" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="TC-10_ExistingDealPayment" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="TC-07_ExistingContactPayment" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="TC-08_SkipLeadPayment" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="TC-09_DirectLeadPayment" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'TC-04_Flow1_NewOrg'!$A$8:$I$33</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'TC-06_ContactsLeadsDeals'!$A$8:$I$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'TC-07_ExistingContactPayment'!$A$8:$I$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'TC-07_ExistingContactPayment'!$A$8:$I$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -605,7 +606,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>tests/Cleanup Scenario.spec.ts, tests/CreateOrganization.spec.ts, tests/Flow1-ExistingOrganization.spec.ts, tests/Flow2-ExistingOrganization.spec.ts, tests/Flow1-NewOrganization.spec.ts, tests/Flow2-NewOrganization.spec.ts, tests/Creating Contacts,Leads,Deals.spec.ts, tests/ExistingContact-ToTenantPayment.spec.ts, tests/Skip lead flow - tenenat Payment.spec.ts, tests/Direct Lead to Tenant Payment.spec.ts</t>
+          <t>tests/Cleanup Scenario.spec.ts, tests/CreateOrganization.spec.ts, tests/Flow1-ExistingOrganization.spec.ts, tests/Flow2-ExistingOrganization.spec.ts, tests/Flow1-NewOrganization.spec.ts, tests/Flow2-NewOrganization.spec.ts, tests/Creating Contacts,Leads,Deals.spec.ts, tests/Existing Deal → Contract → Tenant → Invoice → Receive Payment.spec.ts, tests/Existing Contact → Deal → Contract → Tenant → Invoice → Receive Payment.spec.ts, tests/New Deal → Contract → Tenant → Invoice → Receive Payment.spec.ts, tests/New Lead Creation (Auto-creates Contact) → Deal → Contract → Tenant → Invoice → Receive Payment.spec.ts</t>
         </is>
       </c>
     </row>
@@ -617,7 +618,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>New Org chain: TC-00 Cleanup -&gt; TC-03 CreateOrganization -&gt; TC-04 Flow1-NewOrganization -&gt; TC-06 Creating Contacts,Leads,Deals -&gt; TC-07 ExistingContact-ToTenantPayment -&gt; TC-08 Skip lead flow -&gt; TC-09 Direct Lead to Tenant Payment -&gt; TC-05 Flow2-NewOrganization (optional). Existing org chain: TC-01 Flow1-ExistingOrganization -&gt; TC-02 Flow2-ExistingOrganization.</t>
+          <t>New Org chain: TC-00 Cleanup -&gt; TC-03 CreateOrganization -&gt; TC-04 Flow1-NewOrganization -&gt; TC-06 Creating Contacts,Leads,Deals -&gt; TC-10 Existing Deal -&gt; TC-07 Existing Contact -&gt; Deal -&gt; TC-08 New Deal -&gt; TC-09 New Lead Creation -&gt; TC-05 Flow2-NewOrganization (optional). Existing org chain: TC-01 Flow1-ExistingOrganization -&gt; TC-02 Flow2-ExistingOrganization.</t>
         </is>
       </c>
     </row>
@@ -730,40 +731,51 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TC-07</t>
+          <t>TC-10</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Existing CRM contact -&gt; lead/deal -&gt; tenant -&gt; rent invoice paid. Script: ExistingContact-ToTenantPayment.spec.ts</t>
+          <t>Existing deal (TC-06) -&gt; contract -&gt; tenant -&gt; invoice -&gt; payment. Script: Existing Deal spec</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>TC-08</t>
+          <t>TC-07</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Skip lead: existing contact -&gt; Create Deal -&gt; tenant -&gt; rent payment. Script: Skip lead flow - tenenat Payment.spec.ts</t>
+          <t>Existing CRM contact -&gt; Create Deal (skip lead) -&gt; tenant -&gt; invoice -&gt; payment. Script: Existing Contact spec</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>TC-08</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>New Deal: existing contact -&gt; Create Deal (skip lead) -&gt; tenant -&gt; invoice -&gt; payment. Script: New Deal spec</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>TC-09</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Direct lead: auto contact -&gt; deal -&gt; tenant -&gt; rent payment. Script: Direct Lead to Tenant Payment.spec.ts</t>
-        </is>
-      </c>
-    </row>
-    <row r="23"/>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>New lead (auto contact) -&gt; deal -&gt; contract -&gt; tenant -&gt; invoice -&gt; payment. Script: New Lead Creation (Auto-creates Contact) spec</t>
+        </is>
+      </c>
+    </row>
     <row r="24"/>
     <row r="25"/>
     <row r="26"/>
@@ -782,699 +794,928 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="5" max="5"/>
-    <col width="55" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Skip lead - existing contact Create Deal through rent payment (new org)</t>
-        </is>
-      </c>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="B1" s="16" t="n"/>
+      <c r="C1" s="16" t="n"/>
+      <c r="D1" s="16" t="n"/>
+      <c r="E1" s="16" t="n"/>
+      <c r="F1" s="16" t="n"/>
+      <c r="G1" s="16" t="n"/>
+      <c r="H1" s="16" t="n"/>
+      <c r="I1" s="16" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="16" t="n"/>
+      <c r="B2" s="16" t="n"/>
+      <c r="C2" s="16" t="n"/>
+      <c r="D2" s="16" t="n"/>
+      <c r="E2" s="16" t="n"/>
+      <c r="F2" s="16" t="n"/>
+      <c r="G2" s="16" t="n"/>
+      <c r="H2" s="16" t="n"/>
+      <c r="I2" s="16" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="17" t="inlineStr">
         <is>
           <t>Test ID</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>TC-08</t>
-        </is>
-      </c>
+      <c r="B3" s="16" t="inlineStr">
+        <is>
+          <t>TC-07</t>
+        </is>
+      </c>
+      <c r="C3" s="16" t="n"/>
+      <c r="D3" s="16" t="n"/>
+      <c r="E3" s="16" t="n"/>
+      <c r="F3" s="16" t="n"/>
+      <c r="G3" s="16" t="n"/>
+      <c r="H3" s="16" t="n"/>
+      <c r="I3" s="16" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="n"/>
+      <c r="D4" s="16" t="n"/>
+      <c r="E4" s="16" t="n"/>
+      <c r="F4" s="16" t="n"/>
+      <c r="G4" s="16" t="n"/>
+      <c r="H4" s="16" t="n"/>
+      <c r="I4" s="16" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>End-to-end / Regression</t>
         </is>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="C5" s="16" t="n"/>
+      <c r="D5" s="16" t="n"/>
+      <c r="E5" s="16" t="n"/>
+      <c r="F5" s="16" t="n"/>
+      <c r="G5" s="16" t="n"/>
+      <c r="H5" s="16" t="n"/>
+      <c r="I5" s="16" t="n"/>
+    </row>
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>Precondition</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>TC-03 and TC-06 completed; org.json and crm-contacts-leads.json exist.</t>
-        </is>
-      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>TC-03 and TC-06 completed; test-data/org.json and test-data/crm-contacts-leads.json exist. Deal Approve workflow should already exist from TC-04 (Flow1-NewOrganization).</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="n"/>
+      <c r="D6" s="16" t="n"/>
+      <c r="E6" s="16" t="n"/>
+      <c r="F6" s="16" t="n"/>
+      <c r="G6" s="16" t="n"/>
+      <c r="H6" s="16" t="n"/>
+      <c r="I6" s="16" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Script</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>tests/Skip lead flow - tenenat Payment.spec.ts</t>
-        </is>
-      </c>
+      <c r="A7" s="16" t="n"/>
+      <c r="B7" s="16" t="n"/>
+      <c r="C7" s="16" t="n"/>
+      <c r="D7" s="16" t="n"/>
+      <c r="E7" s="16" t="n"/>
+      <c r="F7" s="16" t="n"/>
+      <c r="G7" s="16" t="n"/>
+      <c r="H7" s="16" t="n"/>
+      <c r="I7" s="16" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>Test ID</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>Step #</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D8" s="9" t="inlineStr">
         <is>
           <t>Actor</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="E8" s="9" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="F8" s="7" t="inlineStr">
+      <c r="F8" s="9" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="G8" s="7" t="inlineStr">
+      <c r="G8" s="9" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="H8" s="7" t="inlineStr">
+      <c r="H8" s="9" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="I8" s="7" t="inlineStr">
+      <c r="I8" s="9" t="inlineStr">
         <is>
           <t>Precondition</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>TC-08</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Skip lead - existing contact Create Deal through rent payment (new org)</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
+    <row r="9" ht="45" customHeight="1">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>TC-07</t>
+        </is>
+      </c>
+      <c r="B9" s="19" t="inlineStr">
+        <is>
+          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Login using orgId, email, password from test-data/org.json</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Admin session starts</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>TC-03 and TC-06 completed; org.json and crm-contacts-leads.json exist.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>TC-08</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Skip lead - existing contact Create Deal through rent payment (new org)</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
+      <c r="D9" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E9" s="19" t="inlineStr">
+        <is>
+          <t>Login using orgId, email, and password from test-data/org.json</t>
+        </is>
+      </c>
+      <c r="F9" s="19" t="inlineStr">
+        <is>
+          <t>Admin session starts after leaving /login</t>
+        </is>
+      </c>
+      <c r="G9" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H9" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I9" s="19" t="inlineStr">
+        <is>
+          <t>TC-03 and TC-06 completed; test-data/org.json and test-data/crm-contacts-leads.json exist. Deal Approve workflow should already exist from TC-04 (Flow1-NewOrganization).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1">
+      <c r="A10" s="19" t="inlineStr">
+        <is>
+          <t>TC-07</t>
+        </is>
+      </c>
+      <c r="B10" s="19" t="inlineStr">
+        <is>
+          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C10" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Configure Razorpay integration and tax settings (GST 18%) if not already done</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Payment and tax setup complete</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>TC-08</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Skip lead - existing contact Create Deal through rent payment (new org)</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
+      <c r="D10" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E10" s="19" t="inlineStr">
+        <is>
+          <t>Open Accounts -&gt; Taxes. Delete VAT if present. Skip create if GST (18%) already exists; otherwise create GST (18%) / GST-18 / 18%</t>
+        </is>
+      </c>
+      <c r="F10" s="19" t="inlineStr">
+        <is>
+          <t>GST (18%) is available in tax dropdowns</t>
+        </is>
+      </c>
+      <c r="G10" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H10" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I10" s="19" t="n"/>
+    </row>
+    <row r="11" ht="45" customHeight="1">
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>TC-07</t>
+        </is>
+      </c>
+      <c r="B11" s="19" t="inlineStr">
+        <is>
+          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C11" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>CRM -&gt; Deals -&gt; Create Deal with shared contact from crm-contacts-leads.json (skip lead creation)</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Deal form opens with contact selected</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>TC-08</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Skip lead - existing contact Create Deal through rent payment (new org)</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
+      <c r="D11" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E11" s="19" t="inlineStr">
+        <is>
+          <t>Go to CRM Contacts and open a random contact from crm-contacts-leads.json</t>
+        </is>
+      </c>
+      <c r="F11" s="19" t="inlineStr">
+        <is>
+          <t>Contact details page opens</t>
+        </is>
+      </c>
+      <c r="G11" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H11" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I11" s="19" t="n"/>
+    </row>
+    <row r="12" ht="45" customHeight="1">
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>TC-07</t>
+        </is>
+      </c>
+      <c r="B12" s="19" t="inlineStr">
+        <is>
+          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C12" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Add vacant property to deal, set rent/discount/GST, mark site visit done</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Deal property pricing saved</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>TC-08</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Skip lead - existing contact Create Deal through rent payment (new org)</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
+      <c r="D12" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E12" s="19" t="inlineStr">
+        <is>
+          <t>Click Create Lead (if lead already exists for this contact, open the existing lead or deal instead)</t>
+        </is>
+      </c>
+      <c r="F12" s="19" t="inlineStr">
+        <is>
+          <t>Lead details or Deal Details page is shown</t>
+        </is>
+      </c>
+      <c r="G12" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H12" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I12" s="19" t="n"/>
+    </row>
+    <row r="13" ht="45" customHeight="1">
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t>TC-07</t>
+        </is>
+      </c>
+      <c r="B13" s="19" t="inlineStr">
+        <is>
+          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C13" s="19" t="n">
         <v>5</v>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Submit for Approval and complete Deal Approve workflow</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Deal is approved</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>TC-08</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Skip lead - existing contact Create Deal through rent payment (new org)</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
+      <c r="D13" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E13" s="19" t="inlineStr">
+        <is>
+          <t>If not already a deal, Convert to Deal and select a payment type</t>
+        </is>
+      </c>
+      <c r="F13" s="19" t="inlineStr">
+        <is>
+          <t>Deal Details page opens</t>
+        </is>
+      </c>
+      <c r="G13" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H13" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I13" s="19" t="n"/>
+    </row>
+    <row r="14" ht="45" customHeight="1">
+      <c r="A14" s="19" t="inlineStr">
+        <is>
+          <t>TC-07</t>
+        </is>
+      </c>
+      <c r="B14" s="19" t="inlineStr">
+        <is>
+          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C14" s="19" t="n">
         <v>6</v>
       </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Create/view contract and approve contract</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Contract approved</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>TC-08</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Skip lead - existing contact Create Deal through rent payment (new org)</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
+      <c r="D14" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E14" s="19" t="inlineStr">
+        <is>
+          <t>If Add Property is enabled, click Add Property. In the dialog set Status combobox to Vacant, select one random vacant property, click Add Property. If Add Property is disabled, keep the property already on the deal</t>
+        </is>
+      </c>
+      <c r="F14" s="19" t="inlineStr">
+        <is>
+          <t>A vacant (or existing) property is on the deal</t>
+        </is>
+      </c>
+      <c r="G14" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H14" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I14" s="19" t="n"/>
+    </row>
+    <row r="15" ht="45" customHeight="1">
+      <c r="A15" s="19" t="inlineStr">
+        <is>
+          <t>TC-07</t>
+        </is>
+      </c>
+      <c r="B15" s="19" t="inlineStr">
+        <is>
+          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C15" s="19" t="n">
         <v>7</v>
       </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Create tenant user; password from dialog or IMAP</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Tenant user created</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>TC-08</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Skip lead - existing contact Create Deal through rent payment (new org)</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
+      <c r="D15" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E15" s="19" t="inlineStr">
+        <is>
+          <t>On the deal property card set Property Rent (120000-600000 if 0), Discount % (10-30), Tax GST (18%), Save, mark Site visit done</t>
+        </is>
+      </c>
+      <c r="F15" s="19" t="inlineStr">
+        <is>
+          <t>Pricing is saved and site visit is done</t>
+        </is>
+      </c>
+      <c r="G15" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H15" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I15" s="19" t="n"/>
+    </row>
+    <row r="16" ht="45" customHeight="1">
+      <c r="A16" s="19" t="inlineStr">
+        <is>
+          <t>TC-07</t>
+        </is>
+      </c>
+      <c r="B16" s="19" t="inlineStr">
+        <is>
+          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C16" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Create move-in request and complete in Operations Requests</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Move-in completed</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>TC-08</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Skip lead - existing contact Create Deal through rent payment (new org)</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
+      <c r="D16" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E16" s="19" t="inlineStr">
+        <is>
+          <t>Click Submit for Approval (confirm dialog if shown), then Approve on Internal Approval and Confirm</t>
+        </is>
+      </c>
+      <c r="F16" s="19" t="inlineStr">
+        <is>
+          <t>Deal approval workflow completes</t>
+        </is>
+      </c>
+      <c r="G16" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H16" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I16" s="19" t="n"/>
+    </row>
+    <row r="17" ht="45" customHeight="1">
+      <c r="A17" s="19" t="inlineStr">
+        <is>
+          <t>TC-07</t>
+        </is>
+      </c>
+      <c r="B17" s="19" t="inlineStr">
+        <is>
+          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C17" s="19" t="n">
         <v>9</v>
       </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
+      <c r="D17" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E17" s="19" t="inlineStr">
+        <is>
+          <t>Create/view contract and approve the contract</t>
+        </is>
+      </c>
+      <c r="F17" s="19" t="inlineStr">
+        <is>
+          <t>Contract is approved</t>
+        </is>
+      </c>
+      <c r="G17" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H17" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I17" s="19" t="n"/>
+    </row>
+    <row r="18" ht="45" customHeight="1">
+      <c r="A18" s="19" t="inlineStr">
+        <is>
+          <t>TC-07</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="inlineStr">
+        <is>
+          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C18" s="19" t="n">
+        <v>10</v>
+      </c>
+      <c r="D18" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E18" s="19" t="inlineStr">
+        <is>
+          <t>Create tenant user from Action Buttons tab</t>
+        </is>
+      </c>
+      <c r="F18" s="19" t="inlineStr">
+        <is>
+          <t>Tenant user is created; password captured from dialog or IMAP (Gmail app password)</t>
+        </is>
+      </c>
+      <c r="G18" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H18" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I18" s="19" t="n"/>
+    </row>
+    <row r="19" ht="45" customHeight="1">
+      <c r="A19" s="19" t="inlineStr">
+        <is>
+          <t>TC-07</t>
+        </is>
+      </c>
+      <c r="B19" s="19" t="inlineStr">
+        <is>
+          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C19" s="19" t="n">
+        <v>11</v>
+      </c>
+      <c r="D19" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E19" s="19" t="inlineStr">
+        <is>
+          <t>Create move-in request with current move-in date; complete it in Operations Requests</t>
+        </is>
+      </c>
+      <c r="F19" s="19" t="inlineStr">
+        <is>
+          <t>Move-in request becomes completed</t>
+        </is>
+      </c>
+      <c r="G19" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H19" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I19" s="19" t="n"/>
+    </row>
+    <row r="20" ht="45" customHeight="1">
+      <c r="A20" s="19" t="inlineStr">
+        <is>
+          <t>TC-07</t>
+        </is>
+      </c>
+      <c r="B20" s="19" t="inlineStr">
+        <is>
+          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C20" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="D20" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E20" s="19" t="inlineStr">
         <is>
           <t>Logout</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Login page displayed</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>TC-08</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Skip lead - existing contact Create Deal through rent payment (new org)</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>10</v>
-      </c>
-      <c r="D18" t="inlineStr">
+      <c r="F20" s="19" t="inlineStr">
+        <is>
+          <t>Login page is displayed</t>
+        </is>
+      </c>
+      <c r="G20" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H20" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I20" s="19" t="n"/>
+    </row>
+    <row r="21" ht="45" customHeight="1">
+      <c r="A21" s="19" t="inlineStr">
+        <is>
+          <t>TC-07</t>
+        </is>
+      </c>
+      <c r="B21" s="19" t="inlineStr">
+        <is>
+          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C21" s="19" t="n">
+        <v>13</v>
+      </c>
+      <c r="D21" s="19" t="inlineStr">
         <is>
           <t>Tenant</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Login with tenant credentials (IMAP or captured password)</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Tenant portal opens</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>TC-08</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Skip lead - existing contact Create Deal through rent payment (new org)</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>11</v>
-      </c>
-      <c r="D19" t="inlineStr">
+      <c r="E21" s="19" t="inlineStr">
+        <is>
+          <t>Login with tenant credentials from IMAP or captured password (orgId from org.json)</t>
+        </is>
+      </c>
+      <c r="F21" s="19" t="inlineStr">
+        <is>
+          <t>Tenant portal opens successfully</t>
+        </is>
+      </c>
+      <c r="G21" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H21" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I21" s="19" t="n"/>
+    </row>
+    <row r="22" ht="45" customHeight="1">
+      <c r="A22" s="19" t="inlineStr">
+        <is>
+          <t>TC-07</t>
+        </is>
+      </c>
+      <c r="B22" s="19" t="inlineStr">
+        <is>
+          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C22" s="19" t="n">
+        <v>14</v>
+      </c>
+      <c r="D22" s="19" t="inlineStr">
         <is>
           <t>Tenant</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E22" s="19" t="inlineStr">
         <is>
           <t>Logout</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Login page displayed</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>TC-08</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Skip lead - existing contact Create Deal through rent payment (new org)</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>12</v>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Create rent invoice (4000 Rental Income), submit/publish</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Invoice visible to tenant</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>TC-08</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Skip lead - existing contact Create Deal through rent payment (new org)</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>13</v>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
+      <c r="F22" s="19" t="inlineStr">
+        <is>
+          <t>Login page is displayed</t>
+        </is>
+      </c>
+      <c r="G22" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H22" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I22" s="19" t="n"/>
+    </row>
+    <row r="23" ht="45" customHeight="1">
+      <c r="A23" s="19" t="inlineStr">
+        <is>
+          <t>TC-07</t>
+        </is>
+      </c>
+      <c r="B23" s="19" t="inlineStr">
+        <is>
+          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C23" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="D23" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E23" s="19" t="inlineStr">
+        <is>
+          <t>Login again and create rent invoice: item rent, Chart of Account 4000 - Rental Income, amount from deal rent; submit/publish</t>
+        </is>
+      </c>
+      <c r="F23" s="19" t="inlineStr">
+        <is>
+          <t>Invoice is due/visible to tenant</t>
+        </is>
+      </c>
+      <c r="G23" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H23" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I23" s="19" t="n"/>
+    </row>
+    <row r="24" ht="45" customHeight="1">
+      <c r="A24" s="19" t="inlineStr">
+        <is>
+          <t>TC-07</t>
+        </is>
+      </c>
+      <c r="B24" s="19" t="inlineStr">
+        <is>
+          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C24" s="19" t="n">
+        <v>16</v>
+      </c>
+      <c r="D24" s="19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E24" s="19" t="inlineStr">
         <is>
           <t>Logout</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Login page displayed</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>TC-08</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Skip lead - existing contact Create Deal through rent payment (new org)</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>14</v>
-      </c>
-      <c r="D22" t="inlineStr">
+      <c r="F24" s="19" t="inlineStr">
+        <is>
+          <t>Login page is displayed</t>
+        </is>
+      </c>
+      <c r="G24" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H24" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I24" s="19" t="n"/>
+    </row>
+    <row r="25" ht="45" customHeight="1">
+      <c r="A25" s="19" t="inlineStr">
+        <is>
+          <t>TC-07</t>
+        </is>
+      </c>
+      <c r="B25" s="19" t="inlineStr">
+        <is>
+          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C25" s="19" t="n">
+        <v>17</v>
+      </c>
+      <c r="D25" s="19" t="inlineStr">
         <is>
           <t>Tenant</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Pay invoice via Razorpay Netbanking -&gt; Bank of Baroda -&gt; Success</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Invoice status PAID</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
+      <c r="E25" s="19" t="inlineStr">
+        <is>
+          <t>Login, open the invoice, Pay Online / Pay with Razorpay, Netbanking -&gt; Bank of Baroda -&gt; Success</t>
+        </is>
+      </c>
+      <c r="F25" s="19" t="inlineStr">
+        <is>
+          <t>Invoice status becomes PAID</t>
+        </is>
+      </c>
+      <c r="G25" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H25" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I25" s="19" t="n"/>
+    </row>
+    <row r="26" ht="45" customHeight="1">
+      <c r="A26" s="19" t="inlineStr">
+        <is>
+          <t>TC-07</t>
+        </is>
+      </c>
+      <c r="B26" s="19" t="inlineStr">
+        <is>
+          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C26" s="19" t="n">
+        <v>18</v>
+      </c>
+      <c r="D26" s="19" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="E26" s="19" t="inlineStr">
+        <is>
+          <t>Save tenant details to test-data/tenant-new-org.json</t>
+        </is>
+      </c>
+      <c r="F26" s="19" t="inlineStr">
+        <is>
+          <t>tenant-new-org.json is updated for optional Flow 2 reuse</t>
+        </is>
+      </c>
+      <c r="G26" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H26" s="19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I26" s="19" t="n"/>
     </row>
   </sheetData>
+  <autoFilter ref="A8:I26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -1497,7 +1738,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Direct Lead - auto contact through rent payment (new org)</t>
+          <t>New Deal - existing contact Create Deal through rent payment (new org)</t>
         </is>
       </c>
     </row>
@@ -1509,7 +1750,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>TC-09</t>
+          <t>TC-08</t>
         </is>
       </c>
     </row>
@@ -1545,7 +1786,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>TC-03 completed; org.json exists with valid Super Admin credentials.</t>
+          <t>TC-03 and TC-06 completed; org.json and crm-contacts-leads.json exist.</t>
         </is>
       </c>
     </row>
@@ -1557,7 +1798,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>tests/Direct Lead to Tenant Payment.spec.ts</t>
+          <t>tests/New Deal → Contract → Tenant → Invoice → Receive Payment.spec.ts</t>
         </is>
       </c>
     </row>
@@ -1611,12 +1852,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TC-09</t>
+          <t>TC-08</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Direct Lead - auto contact through rent payment (new org)</t>
+          <t>New Deal - existing contact Create Deal through rent payment (new org)</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1649,19 +1890,19 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>TC-03 completed; org.json exists with valid Super Admin credentials.</t>
+          <t>TC-03 and TC-06 completed; org.json and crm-contacts-leads.json exist.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TC-09</t>
+          <t>TC-08</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Direct Lead - auto contact through rent payment (new org)</t>
+          <t>New Deal - existing contact Create Deal through rent payment (new org)</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1674,12 +1915,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>CRM -&gt; Leads -&gt; Create New Lead: search tenantN name, No matches -&gt; Create New Lead</t>
+          <t>Configure Razorpay integration and tax settings (GST 18%) if not already done</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Lead create form opens</t>
+          <t>Payment and tax setup complete</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1696,12 +1937,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TC-09</t>
+          <t>TC-08</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Direct Lead - auto contact through rent payment (new org)</t>
+          <t>New Deal - existing contact Create Deal through rent payment (new org)</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1714,12 +1955,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Fill lead form (name, email propexceltest+tenantN@gmail.com, India mobile, nationality), Create</t>
+          <t>CRM -&gt; Deals -&gt; Create Deal with shared contact from crm-contacts-leads.json (skip lead creation)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Lead details page opens (contact auto-created)</t>
+          <t>Deal form opens with contact selected</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1736,12 +1977,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TC-09</t>
+          <t>TC-08</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Direct Lead - auto contact through rent payment (new org)</t>
+          <t>New Deal - existing contact Create Deal through rent payment (new org)</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1754,12 +1995,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Convert to Deal, select payment type</t>
+          <t>Add vacant property to deal, set rent/discount/GST, mark site visit done</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Deal Details page opens</t>
+          <t>Deal property pricing saved</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1776,12 +2017,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TC-09</t>
+          <t>TC-08</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Direct Lead - auto contact through rent payment (new org)</t>
+          <t>New Deal - existing contact Create Deal through rent payment (new org)</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -1794,12 +2035,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Add property to deal, set tax, Approve deal</t>
+          <t>Submit for Approval and complete Deal Approve workflow</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Deal approved</t>
+          <t>Deal is approved</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1816,12 +2057,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TC-09</t>
+          <t>TC-08</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Direct Lead - auto contact through rent payment (new org)</t>
+          <t>New Deal - existing contact Create Deal through rent payment (new org)</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -1856,12 +2097,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>TC-09</t>
+          <t>TC-08</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Direct Lead - auto contact through rent payment (new org)</t>
+          <t>New Deal - existing contact Create Deal through rent payment (new org)</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -1896,12 +2137,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>TC-09</t>
+          <t>TC-08</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Direct Lead - auto contact through rent payment (new org)</t>
+          <t>New Deal - existing contact Create Deal through rent payment (new org)</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -1914,7 +2155,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Create move-in request and complete in Operations</t>
+          <t>Create move-in request and complete in Operations Requests</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1936,12 +2177,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>TC-09</t>
+          <t>TC-08</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Direct Lead - auto contact through rent payment (new org)</t>
+          <t>New Deal - existing contact Create Deal through rent payment (new org)</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -1976,12 +2217,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>TC-09</t>
+          <t>TC-08</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Direct Lead - auto contact through rent payment (new org)</t>
+          <t>New Deal - existing contact Create Deal through rent payment (new org)</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2016,12 +2257,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>TC-09</t>
+          <t>TC-08</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Direct Lead - auto contact through rent payment (new org)</t>
+          <t>New Deal - existing contact Create Deal through rent payment (new org)</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2056,12 +2297,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TC-09</t>
+          <t>TC-08</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Direct Lead - auto contact through rent payment (new org)</t>
+          <t>New Deal - existing contact Create Deal through rent payment (new org)</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2096,12 +2337,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>TC-09</t>
+          <t>TC-08</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Direct Lead - auto contact through rent payment (new org)</t>
+          <t>New Deal - existing contact Create Deal through rent payment (new org)</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2136,12 +2377,712 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>TC-08</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>New Deal - existing contact Create Deal through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>14</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Tenant</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Pay invoice via Razorpay Netbanking -&gt; Bank of Baroda -&gt; Success</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Invoice status PAID</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>New Lead Creation (Auto-creates Contact) - deal through rent payment (new org)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Test ID</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>TC-09</t>
         </is>
       </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>End-to-end / Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>TC-03 completed; org.json exists with valid Super Admin credentials.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Script</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>tests/New Lead Creation (Auto-creates Contact) → Deal → Contract → Tenant → Invoice → Receive Payment.spec.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Test ID</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Step #</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Actor</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TC-09</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>New Lead Creation (Auto-creates Contact) - deal through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Login using orgId, email, password from test-data/org.json</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Admin session starts</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>TC-03 completed; org.json exists with valid Super Admin credentials.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>TC-09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>New Lead Creation (Auto-creates Contact) - deal through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>CRM -&gt; Leads -&gt; Create New Lead: search tenantN name, No matches -&gt; Create New Lead</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Lead create form opens</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TC-09</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>New Lead Creation (Auto-creates Contact) - deal through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>3</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Fill lead form (name, email propexceltest+tenantN@gmail.com, India mobile, nationality), Create</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Lead details page opens (contact auto-created)</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>TC-09</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>New Lead Creation (Auto-creates Contact) - deal through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>4</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Convert to Deal, select payment type</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Deal Details page opens</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>TC-09</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>New Lead Creation (Auto-creates Contact) - deal through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>5</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Add property to deal, set tax, Approve deal</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Deal approved</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>TC-09</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>New Lead Creation (Auto-creates Contact) - deal through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>6</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Create/view contract and approve contract</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Contract approved</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>TC-09</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>New Lead Creation (Auto-creates Contact) - deal through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>7</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Create tenant user; password from dialog or IMAP</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Tenant user created</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>TC-09</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>New Lead Creation (Auto-creates Contact) - deal through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>8</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Create move-in request and complete in Operations</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Move-in completed</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>TC-09</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>New Lead Creation (Auto-creates Contact) - deal through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>9</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Login page displayed</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>TC-09</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>New Lead Creation (Auto-creates Contact) - deal through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Tenant</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Login with tenant credentials (IMAP or captured password)</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Tenant portal opens</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>TC-09</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>New Lead Creation (Auto-creates Contact) - deal through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>11</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Tenant</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Login page displayed</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>TC-09</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>New Lead Creation (Auto-creates Contact) - deal through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>12</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Create rent invoice (4000 Rental Income), submit/publish</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Invoice visible to tenant</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>TC-09</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>New Lead Creation (Auto-creates Contact) - deal through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>13</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Login page displayed</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>TC-09</t>
+        </is>
+      </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Direct Lead - auto contact through rent payment (new org)</t>
+          <t>New Lead Creation (Auto-creates Contact) - deal through rent payment (new org)</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3747,7 +4688,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Login as Super Admin: org test, email test@yopmail.com, password Test2026$</t>
+          <t>Login as Super Admin: org test, email test@gmail.com (propexceltest+tenantN).com, password Test2026$</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -8117,927 +9058,658 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="55" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="15" t="inlineStr">
-        <is>
-          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
-        </is>
-      </c>
-      <c r="B1" s="16" t="n"/>
-      <c r="C1" s="16" t="n"/>
-      <c r="D1" s="16" t="n"/>
-      <c r="E1" s="16" t="n"/>
-      <c r="F1" s="16" t="n"/>
-      <c r="G1" s="16" t="n"/>
-      <c r="H1" s="16" t="n"/>
-      <c r="I1" s="16" t="n"/>
-    </row>
-    <row r="2">
-      <c r="A2" s="16" t="n"/>
-      <c r="B2" s="16" t="n"/>
-      <c r="C2" s="16" t="n"/>
-      <c r="D2" s="16" t="n"/>
-      <c r="E2" s="16" t="n"/>
-      <c r="F2" s="16" t="n"/>
-      <c r="G2" s="16" t="n"/>
-      <c r="H2" s="16" t="n"/>
-      <c r="I2" s="16" t="n"/>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Existing Deal (TC-06) - contract through rent payment (new org)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="17" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Test ID</t>
         </is>
       </c>
-      <c r="B3" s="16" t="inlineStr">
-        <is>
-          <t>TC-07</t>
-        </is>
-      </c>
-      <c r="C3" s="16" t="n"/>
-      <c r="D3" s="16" t="n"/>
-      <c r="E3" s="16" t="n"/>
-      <c r="F3" s="16" t="n"/>
-      <c r="G3" s="16" t="n"/>
-      <c r="H3" s="16" t="n"/>
-      <c r="I3" s="16" t="n"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>TC-10</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="17" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="C4" s="16" t="n"/>
-      <c r="D4" s="16" t="n"/>
-      <c r="E4" s="16" t="n"/>
-      <c r="F4" s="16" t="n"/>
-      <c r="G4" s="16" t="n"/>
-      <c r="H4" s="16" t="n"/>
-      <c r="I4" s="16" t="n"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="17" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>End-to-end / Regression</t>
         </is>
       </c>
-      <c r="C5" s="16" t="n"/>
-      <c r="D5" s="16" t="n"/>
-      <c r="E5" s="16" t="n"/>
-      <c r="F5" s="16" t="n"/>
-      <c r="G5" s="16" t="n"/>
-      <c r="H5" s="16" t="n"/>
-      <c r="I5" s="16" t="n"/>
-    </row>
-    <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="17" t="inlineStr">
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Precondition</t>
         </is>
       </c>
-      <c r="B6" s="18" t="inlineStr">
-        <is>
-          <t>TC-03 and TC-06 completed; test-data/org.json and test-data/crm-contacts-leads.json exist. Deal Approve workflow should already exist from TC-04 (Flow1-NewOrganization).</t>
-        </is>
-      </c>
-      <c r="C6" s="16" t="n"/>
-      <c r="D6" s="16" t="n"/>
-      <c r="E6" s="16" t="n"/>
-      <c r="F6" s="16" t="n"/>
-      <c r="G6" s="16" t="n"/>
-      <c r="H6" s="16" t="n"/>
-      <c r="I6" s="16" t="n"/>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>TC-03, TC-04, and TC-06 completed; org.json and crm-contacts-leads.json exist. GST and Deal Approve workflow already configured by Flow1.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="n"/>
-      <c r="B7" s="16" t="n"/>
-      <c r="C7" s="16" t="n"/>
-      <c r="D7" s="16" t="n"/>
-      <c r="E7" s="16" t="n"/>
-      <c r="F7" s="16" t="n"/>
-      <c r="G7" s="16" t="n"/>
-      <c r="H7" s="16" t="n"/>
-      <c r="I7" s="16" t="n"/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Script</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>tests/Existing Deal → Contract → Tenant → Invoice → Receive Payment.spec.ts</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>Test ID</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>Step #</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
         <is>
           <t>Actor</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="E8" s="7" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="F8" s="9" t="inlineStr">
+      <c r="F8" s="7" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="G8" s="9" t="inlineStr">
+      <c r="G8" s="7" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="H8" s="9" t="inlineStr">
+      <c r="H8" s="7" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="I8" s="9" t="inlineStr">
+      <c r="I8" s="7" t="inlineStr">
         <is>
           <t>Precondition</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="45" customHeight="1">
-      <c r="A9" s="19" t="inlineStr">
-        <is>
-          <t>TC-07</t>
-        </is>
-      </c>
-      <c r="B9" s="19" t="inlineStr">
-        <is>
-          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
-        </is>
-      </c>
-      <c r="C9" s="19" t="n">
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TC-10</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Existing Deal (TC-06) - contract through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
         <v>1</v>
       </c>
-      <c r="D9" s="19" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E9" s="19" t="inlineStr">
-        <is>
-          <t>Login using orgId, email, and password from test-data/org.json</t>
-        </is>
-      </c>
-      <c r="F9" s="19" t="inlineStr">
-        <is>
-          <t>Admin session starts after leaving /login</t>
-        </is>
-      </c>
-      <c r="G9" s="19" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H9" s="19" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I9" s="19" t="inlineStr">
-        <is>
-          <t>TC-03 and TC-06 completed; test-data/org.json and test-data/crm-contacts-leads.json exist. Deal Approve workflow should already exist from TC-04 (Flow1-NewOrganization).</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="45" customHeight="1">
-      <c r="A10" s="19" t="inlineStr">
-        <is>
-          <t>TC-07</t>
-        </is>
-      </c>
-      <c r="B10" s="19" t="inlineStr">
-        <is>
-          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
-        </is>
-      </c>
-      <c r="C10" s="19" t="n">
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Login using orgId, email, password from test-data/org.json</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Admin session starts</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>TC-03, TC-04, and TC-06 completed; org.json and crm-contacts-leads.json exist. GST and Deal Approve workflow already configured by Flow1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>TC-10</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Existing Deal (TC-06) - contract through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
         <v>2</v>
       </c>
-      <c r="D10" s="19" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E10" s="19" t="inlineStr">
-        <is>
-          <t>Open Accounts -&gt; Taxes. Delete VAT if present. Skip create if GST (18%) already exists; otherwise create GST (18%) / GST-18 / 18%</t>
-        </is>
-      </c>
-      <c r="F10" s="19" t="inlineStr">
-        <is>
-          <t>GST (18%) is available in tax dropdowns</t>
-        </is>
-      </c>
-      <c r="G10" s="19" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H10" s="19" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I10" s="19" t="n"/>
-    </row>
-    <row r="11" ht="45" customHeight="1">
-      <c r="A11" s="19" t="inlineStr">
-        <is>
-          <t>TC-07</t>
-        </is>
-      </c>
-      <c r="B11" s="19" t="inlineStr">
-        <is>
-          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
-        </is>
-      </c>
-      <c r="C11" s="19" t="n">
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>CRM -&gt; Deals -&gt; search and open existing deal from crm-contacts-leads.json (TC-06)</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Deal Details page opens</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TC-10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Existing Deal (TC-06) - contract through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
         <v>3</v>
       </c>
-      <c r="D11" s="19" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E11" s="19" t="inlineStr">
-        <is>
-          <t>Go to CRM Contacts and open a random contact from crm-contacts-leads.json</t>
-        </is>
-      </c>
-      <c r="F11" s="19" t="inlineStr">
-        <is>
-          <t>Contact details page opens</t>
-        </is>
-      </c>
-      <c r="G11" s="19" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H11" s="19" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I11" s="19" t="n"/>
-    </row>
-    <row r="12" ht="45" customHeight="1">
-      <c r="A12" s="19" t="inlineStr">
-        <is>
-          <t>TC-07</t>
-        </is>
-      </c>
-      <c r="B12" s="19" t="inlineStr">
-        <is>
-          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
-        </is>
-      </c>
-      <c r="C12" s="19" t="n">
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Add vacant property to deal, set rent/discount/GST, mark site visit done</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Deal property pricing saved</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>TC-10</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Existing Deal (TC-06) - contract through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
         <v>4</v>
       </c>
-      <c r="D12" s="19" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E12" s="19" t="inlineStr">
-        <is>
-          <t>Click Create Lead (if lead already exists for this contact, open the existing lead or deal instead)</t>
-        </is>
-      </c>
-      <c r="F12" s="19" t="inlineStr">
-        <is>
-          <t>Lead details or Deal Details page is shown</t>
-        </is>
-      </c>
-      <c r="G12" s="19" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H12" s="19" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I12" s="19" t="n"/>
-    </row>
-    <row r="13" ht="45" customHeight="1">
-      <c r="A13" s="19" t="inlineStr">
-        <is>
-          <t>TC-07</t>
-        </is>
-      </c>
-      <c r="B13" s="19" t="inlineStr">
-        <is>
-          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
-        </is>
-      </c>
-      <c r="C13" s="19" t="n">
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Submit for Approval and complete Deal Approve workflow</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Deal is approved</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>TC-10</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Existing Deal (TC-06) - contract through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
         <v>5</v>
       </c>
-      <c r="D13" s="19" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E13" s="19" t="inlineStr">
-        <is>
-          <t>If not already a deal, Convert to Deal and select a payment type</t>
-        </is>
-      </c>
-      <c r="F13" s="19" t="inlineStr">
-        <is>
-          <t>Deal Details page opens</t>
-        </is>
-      </c>
-      <c r="G13" s="19" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H13" s="19" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I13" s="19" t="n"/>
-    </row>
-    <row r="14" ht="45" customHeight="1">
-      <c r="A14" s="19" t="inlineStr">
-        <is>
-          <t>TC-07</t>
-        </is>
-      </c>
-      <c r="B14" s="19" t="inlineStr">
-        <is>
-          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
-        </is>
-      </c>
-      <c r="C14" s="19" t="n">
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Create/view contract and approve contract</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Contract approved</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>TC-10</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Existing Deal (TC-06) - contract through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
         <v>6</v>
       </c>
-      <c r="D14" s="19" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E14" s="19" t="inlineStr">
-        <is>
-          <t>If Add Property is enabled, click Add Property. In the dialog set Status combobox to Vacant, select one random vacant property, click Add Property. If Add Property is disabled, keep the property already on the deal</t>
-        </is>
-      </c>
-      <c r="F14" s="19" t="inlineStr">
-        <is>
-          <t>A vacant (or existing) property is on the deal</t>
-        </is>
-      </c>
-      <c r="G14" s="19" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H14" s="19" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I14" s="19" t="n"/>
-    </row>
-    <row r="15" ht="45" customHeight="1">
-      <c r="A15" s="19" t="inlineStr">
-        <is>
-          <t>TC-07</t>
-        </is>
-      </c>
-      <c r="B15" s="19" t="inlineStr">
-        <is>
-          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
-        </is>
-      </c>
-      <c r="C15" s="19" t="n">
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Create tenant user; password from dialog or IMAP</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Tenant user created</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>TC-10</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Existing Deal (TC-06) - contract through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
         <v>7</v>
       </c>
-      <c r="D15" s="19" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E15" s="19" t="inlineStr">
-        <is>
-          <t>On the deal property card set Property Rent (120000-600000 if 0), Discount % (10-30), Tax GST (18%), Save, mark Site visit done</t>
-        </is>
-      </c>
-      <c r="F15" s="19" t="inlineStr">
-        <is>
-          <t>Pricing is saved and site visit is done</t>
-        </is>
-      </c>
-      <c r="G15" s="19" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H15" s="19" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I15" s="19" t="n"/>
-    </row>
-    <row r="16" ht="45" customHeight="1">
-      <c r="A16" s="19" t="inlineStr">
-        <is>
-          <t>TC-07</t>
-        </is>
-      </c>
-      <c r="B16" s="19" t="inlineStr">
-        <is>
-          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
-        </is>
-      </c>
-      <c r="C16" s="19" t="n">
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Create move-in request and complete in Operations Requests</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Move-in completed</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>TC-10</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Existing Deal (TC-06) - contract through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
         <v>8</v>
       </c>
-      <c r="D16" s="19" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E16" s="19" t="inlineStr">
-        <is>
-          <t>Click Submit for Approval (confirm dialog if shown), then Approve on Internal Approval and Confirm</t>
-        </is>
-      </c>
-      <c r="F16" s="19" t="inlineStr">
-        <is>
-          <t>Deal approval workflow completes</t>
-        </is>
-      </c>
-      <c r="G16" s="19" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H16" s="19" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I16" s="19" t="n"/>
-    </row>
-    <row r="17" ht="45" customHeight="1">
-      <c r="A17" s="19" t="inlineStr">
-        <is>
-          <t>TC-07</t>
-        </is>
-      </c>
-      <c r="B17" s="19" t="inlineStr">
-        <is>
-          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
-        </is>
-      </c>
-      <c r="C17" s="19" t="n">
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Login page displayed</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>TC-10</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Existing Deal (TC-06) - contract through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
         <v>9</v>
       </c>
-      <c r="D17" s="19" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E17" s="19" t="inlineStr">
-        <is>
-          <t>Create/view contract and approve the contract</t>
-        </is>
-      </c>
-      <c r="F17" s="19" t="inlineStr">
-        <is>
-          <t>Contract is approved</t>
-        </is>
-      </c>
-      <c r="G17" s="19" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H17" s="19" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I17" s="19" t="n"/>
-    </row>
-    <row r="18" ht="45" customHeight="1">
-      <c r="A18" s="19" t="inlineStr">
-        <is>
-          <t>TC-07</t>
-        </is>
-      </c>
-      <c r="B18" s="19" t="inlineStr">
-        <is>
-          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
-        </is>
-      </c>
-      <c r="C18" s="19" t="n">
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Tenant</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Login with tenant credentials (IMAP or captured password)</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Tenant portal opens</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>TC-10</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Existing Deal (TC-06) - contract through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
         <v>10</v>
       </c>
-      <c r="D18" s="19" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E18" s="19" t="inlineStr">
-        <is>
-          <t>Create tenant user from Action Buttons tab</t>
-        </is>
-      </c>
-      <c r="F18" s="19" t="inlineStr">
-        <is>
-          <t>Tenant user is created; password captured from dialog or IMAP (Gmail app password)</t>
-        </is>
-      </c>
-      <c r="G18" s="19" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H18" s="19" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I18" s="19" t="n"/>
-    </row>
-    <row r="19" ht="45" customHeight="1">
-      <c r="A19" s="19" t="inlineStr">
-        <is>
-          <t>TC-07</t>
-        </is>
-      </c>
-      <c r="B19" s="19" t="inlineStr">
-        <is>
-          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
-        </is>
-      </c>
-      <c r="C19" s="19" t="n">
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Tenant</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Login page displayed</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>TC-10</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Existing Deal (TC-06) - contract through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
         <v>11</v>
       </c>
-      <c r="D19" s="19" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E19" s="19" t="inlineStr">
-        <is>
-          <t>Create move-in request with current move-in date; complete it in Operations Requests</t>
-        </is>
-      </c>
-      <c r="F19" s="19" t="inlineStr">
-        <is>
-          <t>Move-in request becomes completed</t>
-        </is>
-      </c>
-      <c r="G19" s="19" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H19" s="19" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I19" s="19" t="n"/>
-    </row>
-    <row r="20" ht="45" customHeight="1">
-      <c r="A20" s="19" t="inlineStr">
-        <is>
-          <t>TC-07</t>
-        </is>
-      </c>
-      <c r="B20" s="19" t="inlineStr">
-        <is>
-          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
-        </is>
-      </c>
-      <c r="C20" s="19" t="n">
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Create rent invoice (4000 Rental Income), submit/publish</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Invoice visible to tenant</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>TC-10</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Existing Deal (TC-06) - contract through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
         <v>12</v>
       </c>
-      <c r="D20" s="19" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E20" s="19" t="inlineStr">
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
         <is>
           <t>Logout</t>
         </is>
       </c>
-      <c r="F20" s="19" t="inlineStr">
-        <is>
-          <t>Login page is displayed</t>
-        </is>
-      </c>
-      <c r="G20" s="19" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H20" s="19" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I20" s="19" t="n"/>
-    </row>
-    <row r="21" ht="45" customHeight="1">
-      <c r="A21" s="19" t="inlineStr">
-        <is>
-          <t>TC-07</t>
-        </is>
-      </c>
-      <c r="B21" s="19" t="inlineStr">
-        <is>
-          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
-        </is>
-      </c>
-      <c r="C21" s="19" t="n">
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Login page displayed</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>TC-10</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Existing Deal (TC-06) - contract through rent payment (new org)</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
         <v>13</v>
       </c>
-      <c r="D21" s="19" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>Tenant</t>
         </is>
       </c>
-      <c r="E21" s="19" t="inlineStr">
-        <is>
-          <t>Login with tenant credentials from IMAP or captured password (orgId from org.json)</t>
-        </is>
-      </c>
-      <c r="F21" s="19" t="inlineStr">
-        <is>
-          <t>Tenant portal opens successfully</t>
-        </is>
-      </c>
-      <c r="G21" s="19" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H21" s="19" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I21" s="19" t="n"/>
-    </row>
-    <row r="22" ht="45" customHeight="1">
-      <c r="A22" s="19" t="inlineStr">
-        <is>
-          <t>TC-07</t>
-        </is>
-      </c>
-      <c r="B22" s="19" t="inlineStr">
-        <is>
-          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
-        </is>
-      </c>
-      <c r="C22" s="19" t="n">
-        <v>14</v>
-      </c>
-      <c r="D22" s="19" t="inlineStr">
-        <is>
-          <t>Tenant</t>
-        </is>
-      </c>
-      <c r="E22" s="19" t="inlineStr">
-        <is>
-          <t>Logout</t>
-        </is>
-      </c>
-      <c r="F22" s="19" t="inlineStr">
-        <is>
-          <t>Login page is displayed</t>
-        </is>
-      </c>
-      <c r="G22" s="19" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H22" s="19" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I22" s="19" t="n"/>
-    </row>
-    <row r="23" ht="45" customHeight="1">
-      <c r="A23" s="19" t="inlineStr">
-        <is>
-          <t>TC-07</t>
-        </is>
-      </c>
-      <c r="B23" s="19" t="inlineStr">
-        <is>
-          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
-        </is>
-      </c>
-      <c r="C23" s="19" t="n">
-        <v>15</v>
-      </c>
-      <c r="D23" s="19" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E23" s="19" t="inlineStr">
-        <is>
-          <t>Login again and create rent invoice: item rent, Chart of Account 4000 - Rental Income, amount from deal rent; submit/publish</t>
-        </is>
-      </c>
-      <c r="F23" s="19" t="inlineStr">
-        <is>
-          <t>Invoice is due/visible to tenant</t>
-        </is>
-      </c>
-      <c r="G23" s="19" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H23" s="19" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I23" s="19" t="n"/>
-    </row>
-    <row r="24" ht="45" customHeight="1">
-      <c r="A24" s="19" t="inlineStr">
-        <is>
-          <t>TC-07</t>
-        </is>
-      </c>
-      <c r="B24" s="19" t="inlineStr">
-        <is>
-          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
-        </is>
-      </c>
-      <c r="C24" s="19" t="n">
-        <v>16</v>
-      </c>
-      <c r="D24" s="19" t="inlineStr">
-        <is>
-          <t>Super Admin</t>
-        </is>
-      </c>
-      <c r="E24" s="19" t="inlineStr">
-        <is>
-          <t>Logout</t>
-        </is>
-      </c>
-      <c r="F24" s="19" t="inlineStr">
-        <is>
-          <t>Login page is displayed</t>
-        </is>
-      </c>
-      <c r="G24" s="19" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H24" s="19" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I24" s="19" t="n"/>
-    </row>
-    <row r="25" ht="45" customHeight="1">
-      <c r="A25" s="19" t="inlineStr">
-        <is>
-          <t>TC-07</t>
-        </is>
-      </c>
-      <c r="B25" s="19" t="inlineStr">
-        <is>
-          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
-        </is>
-      </c>
-      <c r="C25" s="19" t="n">
-        <v>17</v>
-      </c>
-      <c r="D25" s="19" t="inlineStr">
-        <is>
-          <t>Tenant</t>
-        </is>
-      </c>
-      <c r="E25" s="19" t="inlineStr">
-        <is>
-          <t>Login, open the invoice, Pay Online / Pay with Razorpay, Netbanking -&gt; Bank of Baroda -&gt; Success</t>
-        </is>
-      </c>
-      <c r="F25" s="19" t="inlineStr">
-        <is>
-          <t>Invoice status becomes PAID</t>
-        </is>
-      </c>
-      <c r="G25" s="19" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H25" s="19" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I25" s="19" t="n"/>
-    </row>
-    <row r="26" ht="45" customHeight="1">
-      <c r="A26" s="19" t="inlineStr">
-        <is>
-          <t>TC-07</t>
-        </is>
-      </c>
-      <c r="B26" s="19" t="inlineStr">
-        <is>
-          <t>Existing Contact to Tenant Payment - onboard contact through rent payment (new org)</t>
-        </is>
-      </c>
-      <c r="C26" s="19" t="n">
-        <v>18</v>
-      </c>
-      <c r="D26" s="19" t="inlineStr">
-        <is>
-          <t>System</t>
-        </is>
-      </c>
-      <c r="E26" s="19" t="inlineStr">
-        <is>
-          <t>Save tenant details to test-data/tenant-new-org.json</t>
-        </is>
-      </c>
-      <c r="F26" s="19" t="inlineStr">
-        <is>
-          <t>tenant-new-org.json is updated for optional Flow 2 reuse</t>
-        </is>
-      </c>
-      <c r="G26" s="19" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H26" s="19" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="I26" s="19" t="n"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Pay invoice via Razorpay Netbanking -&gt; Bank of Baroda -&gt; Success</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Invoice status PAID</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A8:I26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>